<commit_message>
Daily attendance update - 2026-03-02
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7EBD9B-4054-451E-A0B6-167931150A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E25791-FCA0-4277-9238-058D58E93356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="13" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="UV-WMS Admin December 2025" sheetId="12" r:id="rId12"/>
     <sheet name="UV-WMS Admin January 2026" sheetId="13" r:id="rId13"/>
     <sheet name="UV-WMS Admin February 2026" sheetId="14" r:id="rId14"/>
+    <sheet name="UV-WMS Admin March 2026" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2080" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -360,7 +361,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="37">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1032,31 +1063,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1166,7 +1197,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1266,7 +1297,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1360,7 +1391,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1454,7 +1485,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1548,7 +1579,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1642,7 +1673,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1736,7 +1767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1747,7 +1778,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1760,7 +1791,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1773,7 +1804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1786,7 +1817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1799,7 +1830,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1828,30 +1859,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1961,7 +1992,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2061,7 +2092,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2155,7 +2186,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2249,7 +2280,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2343,7 +2374,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2437,7 +2468,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2475,7 +2506,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2486,7 +2517,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2499,7 +2530,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2512,7 +2543,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2525,7 +2556,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2548,13 +2579,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2565,26 +2596,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2691,7 +2722,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2788,7 +2819,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2875,7 +2906,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2962,7 +2993,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3049,7 +3080,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3136,7 +3167,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3173,7 +3204,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3184,7 +3215,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3197,7 +3228,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3210,7 +3241,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3223,7 +3254,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3246,13 +3277,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3263,27 +3294,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3393,7 +3424,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3493,7 +3524,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3587,7 +3618,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3681,7 +3712,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3775,7 +3806,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3869,7 +3900,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3907,7 +3938,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3918,7 +3949,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3931,7 +3962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3944,7 +3975,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3957,7 +3988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3980,13 +4011,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3997,27 +4028,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4127,7 +4158,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4227,7 +4258,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4319,7 +4350,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4411,7 +4442,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4503,7 +4534,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4595,7 +4626,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4633,7 +4664,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4644,7 +4675,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4657,7 +4688,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4670,7 +4701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4683,7 +4714,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4706,13 +4737,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4723,26 +4754,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4843,7 +4874,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4934,7 +4965,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5019,7 +5050,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5104,7 +5135,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5189,7 +5220,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5274,7 +5305,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5309,7 +5340,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5320,7 +5351,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5333,7 +5364,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5346,7 +5377,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5359,7 +5390,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5370,6 +5401,563 @@
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
         <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B12:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
+  <dimension ref="A1:AJ15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46082</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46083</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46084</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46085</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46086</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46087</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46088</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46089</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46090</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46091</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46092</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46093</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46094</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46095</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46096</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46097</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46098</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46099</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46100</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46101</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46102</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46103</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46104</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46105</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46106</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46107</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46108</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46109</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46110</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46111</v>
+      </c>
+      <c r="AJ1" s="1">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="7"/>
+      <c r="G3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="7"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="7"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="7"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="2"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="7"/>
+      <c r="G5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="7"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="7"/>
+      <c r="AI5" s="2"/>
+      <c r="AJ5" s="2"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="7"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="7"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="7"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2"/>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF(F3:AG3,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIF(F3:AG3,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F4:AG4,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(F4:AG4,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F5:AG5,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F6:AG6,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(F6:AG6,"WFH")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5400,30 +5988,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5524,7 +6112,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5615,7 +6203,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5700,7 +6288,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5787,7 +6375,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5874,7 +6462,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -5959,7 +6547,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -6044,7 +6632,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -6055,7 +6643,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -6068,7 +6656,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -6081,7 +6669,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -6094,7 +6682,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -6107,7 +6695,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6136,28 +6724,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6267,7 +6855,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6367,7 +6955,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6457,7 +7045,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6545,7 +7133,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6633,7 +7221,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6721,7 +7309,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6759,7 +7347,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -6770,7 +7358,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6783,7 +7371,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6796,7 +7384,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6809,7 +7397,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -6832,10 +7420,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="33" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="36" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6847,29 +7435,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6976,7 +7564,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7073,7 +7661,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7164,7 +7752,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7255,7 +7843,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7346,7 +7934,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7437,7 +8025,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7474,7 +8062,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -7485,7 +8073,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -7498,7 +8086,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -7511,7 +8099,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -7524,7 +8112,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -7547,10 +8135,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="31" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7562,29 +8150,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7694,7 +8282,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7794,7 +8382,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7886,7 +8474,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7978,7 +8566,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8070,7 +8658,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8162,7 +8750,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8199,7 +8787,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8210,7 +8798,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8223,7 +8811,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8236,7 +8824,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8249,7 +8837,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8272,15 +8860,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="29" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8291,15 +8879,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8406,7 +8994,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8503,7 +9091,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8592,7 +9180,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8681,7 +9269,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8770,7 +9358,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8859,7 +9447,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8896,7 +9484,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -8907,7 +9495,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -8920,7 +9508,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -8933,7 +9521,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -8946,7 +9534,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -8969,13 +9557,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8986,17 +9574,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9106,7 +9694,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9206,7 +9794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9300,7 +9888,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9394,7 +9982,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9488,7 +10076,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9582,7 +10170,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9619,7 +10207,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -9630,7 +10218,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -9643,7 +10231,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -9656,7 +10244,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -9669,7 +10257,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9692,13 +10280,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9709,18 +10297,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9831,7 +10419,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9931,7 +10519,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10021,7 +10609,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10111,7 +10699,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10201,7 +10789,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10291,7 +10879,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10329,7 +10917,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -10340,7 +10928,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10353,7 +10941,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10366,7 +10954,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -10379,7 +10967,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -10402,13 +10990,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10419,19 +11007,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10538,7 +11126,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10635,7 +11223,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10726,7 +11314,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10817,7 +11405,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10908,7 +11496,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10999,7 +11587,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11036,7 +11624,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11047,7 +11635,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11060,7 +11648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11073,7 +11661,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11086,7 +11674,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11109,13 +11697,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-03
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E25791-FCA0-4277-9238-058D58E93356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B334687-1988-4E53-8B8C-D917EDF8D6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2143" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2147" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5679,7 +5679,9 @@
       <c r="G3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
@@ -5729,7 +5731,9 @@
       <c r="G4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -5779,7 +5783,9 @@
       <c r="G5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -5829,7 +5835,9 @@
       <c r="G6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -5914,7 +5922,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -5927,7 +5935,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -5940,7 +5948,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -5953,7 +5961,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-04
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B334687-1988-4E53-8B8C-D917EDF8D6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE1BFFF-1D2E-4AFB-BBE1-0E4509FEE650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2147" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2159" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5682,9 +5682,15 @@
       <c r="H3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
+      <c r="I3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
       <c r="N3" s="2"/>
@@ -5734,9 +5740,15 @@
       <c r="H4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
+      <c r="I4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="2"/>
@@ -5786,9 +5798,15 @@
       <c r="H5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="I5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
       <c r="N5" s="2"/>
@@ -5838,9 +5856,15 @@
       <c r="H6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="I6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="2"/>
@@ -5922,11 +5946,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -5935,11 +5959,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -5948,11 +5972,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -5961,11 +5985,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-10
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE1BFFF-1D2E-4AFB-BBE1-0E4509FEE650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5BC3F6-0D95-4FA9-98CE-928D4CBC32AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2159" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2165" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -1063,31 +1063,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1197,7 +1197,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1297,7 +1297,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1830,7 +1830,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1859,30 +1859,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2092,7 +2092,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2506,7 +2506,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2517,7 +2517,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2556,7 +2556,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2596,26 +2596,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2819,7 +2819,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2906,7 +2906,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2993,7 +2993,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3080,7 +3080,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3167,7 +3167,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3204,7 +3204,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3294,27 +3294,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3524,7 +3524,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3938,7 +3938,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3949,7 +3949,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3962,7 +3962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4028,27 +4028,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4258,7 +4258,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4664,7 +4664,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4701,7 +4701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4754,26 +4754,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4874,7 +4874,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4965,7 +4965,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5305,7 +5305,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5340,7 +5340,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5351,7 +5351,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5364,7 +5364,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5377,7 +5377,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5390,7 +5390,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5430,26 +5430,26 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5559,7 +5559,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5659,7 +5659,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5693,8 +5693,12 @@
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="N3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
@@ -5717,7 +5721,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5751,8 +5755,12 @@
       </c>
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="N4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
@@ -5775,7 +5783,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5809,7 +5817,9 @@
       </c>
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
-      <c r="N5" s="2"/>
+      <c r="N5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -5833,7 +5843,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5867,7 +5877,9 @@
       </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
-      <c r="N6" s="2"/>
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
@@ -5891,7 +5903,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5929,7 +5941,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5940,52 +5952,52 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -6020,30 +6032,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6144,7 +6156,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6235,7 +6247,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6320,7 +6332,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6407,7 +6419,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6494,7 +6506,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -6579,7 +6591,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -6664,7 +6676,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -6675,7 +6687,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -6688,7 +6700,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -6701,7 +6713,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -6714,7 +6726,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -6727,7 +6739,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6756,28 +6768,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6887,7 +6899,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6987,7 +6999,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7077,7 +7089,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7165,7 +7177,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7253,7 +7265,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7341,7 +7353,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7379,7 +7391,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -7390,7 +7402,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -7403,7 +7415,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -7416,7 +7428,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -7429,7 +7441,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -7467,29 +7479,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7596,7 +7608,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7693,7 +7705,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7784,7 +7796,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7875,7 +7887,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7966,7 +7978,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8057,7 +8069,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8094,7 +8106,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8105,7 +8117,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8118,7 +8130,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8131,7 +8143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8144,7 +8156,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8182,29 +8194,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8314,7 +8326,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8414,7 +8426,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8506,7 +8518,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8598,7 +8610,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8690,7 +8702,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8782,7 +8794,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8819,7 +8831,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8830,7 +8842,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8843,7 +8855,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8856,7 +8868,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8869,7 +8881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8911,15 +8923,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9026,7 +9038,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9123,7 +9135,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9212,7 +9224,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9301,7 +9313,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9390,7 +9402,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9479,7 +9491,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9516,7 +9528,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -9527,7 +9539,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -9540,7 +9552,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -9553,7 +9565,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -9566,7 +9578,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9606,17 +9618,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9726,7 +9738,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9826,7 +9838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9920,7 +9932,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10014,7 +10026,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10108,7 +10120,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10202,7 +10214,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10239,7 +10251,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -10250,7 +10262,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10263,7 +10275,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10276,7 +10288,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -10289,7 +10301,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -10329,18 +10341,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10451,7 +10463,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10551,7 +10563,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10641,7 +10653,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10731,7 +10743,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10821,7 +10833,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10911,7 +10923,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10949,7 +10961,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -10960,7 +10972,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10973,7 +10985,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10986,7 +10998,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -10999,7 +11011,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11039,19 +11051,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11158,7 +11170,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11255,7 +11267,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11346,7 +11358,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11437,7 +11449,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11528,7 +11540,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11619,7 +11631,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11656,7 +11668,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11667,7 +11679,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11680,7 +11692,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11693,7 +11705,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11706,7 +11718,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-11
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5BC3F6-0D95-4FA9-98CE-928D4CBC32AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F539B9-9A7C-4758-AD1E-9AE974AF27C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2165" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2171" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -1063,31 +1063,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1197,7 +1197,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1297,7 +1297,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1830,7 +1830,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1859,30 +1859,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1992,7 +1992,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2092,7 +2092,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2506,7 +2506,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2517,7 +2517,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2556,7 +2556,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2596,26 +2596,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2819,7 +2819,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2906,7 +2906,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2993,7 +2993,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3080,7 +3080,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3167,7 +3167,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3204,7 +3204,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3294,27 +3294,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3524,7 +3524,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3900,7 +3900,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3938,7 +3938,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3949,7 +3949,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3962,7 +3962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3988,7 +3988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4028,27 +4028,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4258,7 +4258,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4664,7 +4664,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4688,7 +4688,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4701,7 +4701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4754,26 +4754,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4874,7 +4874,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4965,7 +4965,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5305,7 +5305,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5340,7 +5340,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5351,7 +5351,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5364,7 +5364,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5377,7 +5377,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5390,7 +5390,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5430,26 +5430,26 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5559,7 +5559,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5659,7 +5659,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5699,7 +5699,9 @@
       <c r="O3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P3" s="2"/>
+      <c r="P3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="7"/>
@@ -5721,7 +5723,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5761,7 +5763,9 @@
       <c r="O4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="2"/>
+      <c r="P4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
       <c r="S4" s="7"/>
@@ -5783,7 +5787,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5820,8 +5824,12 @@
       <c r="N5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
+      <c r="O5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
       <c r="S5" s="7"/>
@@ -5843,7 +5851,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5880,8 +5888,12 @@
       <c r="N6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
+      <c r="O6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
       <c r="S6" s="7"/>
@@ -5903,7 +5915,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5941,7 +5953,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5952,52 +5964,52 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -6032,30 +6044,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6156,7 +6168,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6247,7 +6259,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6332,7 +6344,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6419,7 +6431,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6506,7 +6518,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -6591,7 +6603,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -6676,7 +6688,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -6687,7 +6699,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -6700,7 +6712,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -6713,7 +6725,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -6726,7 +6738,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -6739,7 +6751,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6768,28 +6780,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6899,7 +6911,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6999,7 +7011,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7089,7 +7101,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7177,7 +7189,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7265,7 +7277,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7353,7 +7365,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7391,7 +7403,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -7402,7 +7414,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -7415,7 +7427,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -7428,7 +7440,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -7441,7 +7453,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -7479,29 +7491,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7608,7 +7620,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7705,7 +7717,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7796,7 +7808,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7887,7 +7899,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7978,7 +7990,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8069,7 +8081,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8106,7 +8118,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8117,7 +8129,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8130,7 +8142,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8143,7 +8155,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8156,7 +8168,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8194,29 +8206,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8326,7 +8338,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8426,7 +8438,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8518,7 +8530,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8610,7 +8622,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8702,7 +8714,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8794,7 +8806,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8831,7 +8843,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8842,7 +8854,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8855,7 +8867,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8868,7 +8880,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8881,7 +8893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8923,15 +8935,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9038,7 +9050,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9135,7 +9147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9224,7 +9236,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9313,7 +9325,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9402,7 +9414,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9491,7 +9503,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9528,7 +9540,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -9539,7 +9551,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -9552,7 +9564,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -9565,7 +9577,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -9578,7 +9590,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9618,17 +9630,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9738,7 +9750,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9838,7 +9850,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9932,7 +9944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10026,7 +10038,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10120,7 +10132,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10214,7 +10226,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10251,7 +10263,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -10262,7 +10274,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10275,7 +10287,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10288,7 +10300,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -10301,7 +10313,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -10341,18 +10353,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10463,7 +10475,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10563,7 +10575,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10653,7 +10665,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10743,7 +10755,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10833,7 +10845,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10923,7 +10935,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10961,7 +10973,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -10972,7 +10984,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10985,7 +10997,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10998,7 +11010,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11011,7 +11023,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11051,19 +11063,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11170,7 +11182,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11267,7 +11279,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11358,7 +11370,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11449,7 +11461,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11540,7 +11552,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11631,7 +11643,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11668,7 +11680,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11679,7 +11691,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11692,7 +11704,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11705,7 +11717,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11718,7 +11730,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-12
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F539B9-9A7C-4758-AD1E-9AE974AF27C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1CE8CE-01C1-4D01-B9AD-814F50ADAF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2171" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2181" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5702,14 +5702,20 @@
       <c r="P3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
+      <c r="Q3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="S3" s="7"/>
       <c r="T3" s="7"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
+      <c r="X3" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="Y3" s="2"/>
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
@@ -5766,15 +5772,21 @@
       <c r="P4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
+      <c r="Q4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="S4" s="7"/>
       <c r="T4" s="7"/>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
+      <c r="Y4" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="Z4" s="7"/>
       <c r="AA4" s="7"/>
       <c r="AB4" s="2"/>
@@ -5830,8 +5842,12 @@
       <c r="P5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
+      <c r="Q5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="S5" s="7"/>
       <c r="T5" s="7"/>
       <c r="U5" s="2"/>
@@ -5894,8 +5910,12 @@
       <c r="P6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
+      <c r="Q6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="S6" s="7"/>
       <c r="T6" s="7"/>
       <c r="U6" s="2"/>
@@ -5974,7 +5994,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -5987,7 +6007,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -6000,7 +6020,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -6013,7 +6033,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-13
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1CE8CE-01C1-4D01-B9AD-814F50ADAF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B8ADF5-6F68-478D-A9D1-60C0FBA8700D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -5910,11 +5910,11 @@
       <c r="P6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>17</v>
+      <c r="Q6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="S6" s="7"/>
       <c r="T6" s="7"/>
@@ -6029,11 +6029,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-16
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B8ADF5-6F68-478D-A9D1-60C0FBA8700D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12736EDF-2810-41AB-A53E-5742CB6EA1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2181" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2185" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5710,7 +5710,9 @@
       </c>
       <c r="S3" s="7"/>
       <c r="T3" s="7"/>
-      <c r="U3" s="2"/>
+      <c r="U3" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
       <c r="X3" s="6" t="s">
@@ -5780,7 +5782,9 @@
       </c>
       <c r="S4" s="7"/>
       <c r="T4" s="7"/>
-      <c r="U4" s="2"/>
+      <c r="U4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
@@ -5850,7 +5854,9 @@
       </c>
       <c r="S5" s="7"/>
       <c r="T5" s="7"/>
-      <c r="U5" s="2"/>
+      <c r="U5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
@@ -5918,7 +5924,9 @@
       </c>
       <c r="S6" s="7"/>
       <c r="T6" s="7"/>
-      <c r="U6" s="2"/>
+      <c r="U6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
@@ -6003,7 +6011,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6016,7 +6024,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6029,7 +6037,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-17
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12736EDF-2810-41AB-A53E-5742CB6EA1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2C1AF1-380C-47F9-9016-9D40472CC5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2185" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2189" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5713,7 +5713,9 @@
       <c r="U3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="2"/>
+      <c r="V3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W3" s="2"/>
       <c r="X3" s="6" t="s">
         <v>24</v>
@@ -5785,7 +5787,9 @@
       <c r="U4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="V4" s="2"/>
+      <c r="V4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
       <c r="Y4" s="6" t="s">
@@ -5857,7 +5861,9 @@
       <c r="U5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="V5" s="2"/>
+      <c r="V5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
       <c r="Y5" s="2"/>
@@ -5927,7 +5933,9 @@
       <c r="U6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="V6" s="2"/>
+      <c r="V6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
@@ -5998,7 +6006,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6011,7 +6019,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6028,7 +6036,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -6037,7 +6045,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-23
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2C1AF1-380C-47F9-9016-9D40472CC5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC7AA83-347F-4963-8DFC-BB66E13E1DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2189" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2203" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5716,14 +5716,20 @@
       <c r="V3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="W3" s="2"/>
+      <c r="W3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="X3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Y3" s="2"/>
+      <c r="Y3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
-      <c r="AB3" s="2"/>
+      <c r="AB3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
@@ -5790,14 +5796,20 @@
       <c r="V4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
+      <c r="W4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Y4" s="6" t="s">
         <v>24</v>
       </c>
       <c r="Z4" s="7"/>
       <c r="AA4" s="7"/>
-      <c r="AB4" s="2"/>
+      <c r="AB4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC4" s="2"/>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
@@ -5864,12 +5876,20 @@
       <c r="V5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
+      <c r="W5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Z5" s="7"/>
       <c r="AA5" s="7"/>
-      <c r="AB5" s="2"/>
+      <c r="AB5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
@@ -5936,12 +5956,20 @@
       <c r="V6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
+      <c r="W6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
-      <c r="AB6" s="2"/>
+      <c r="AB6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
@@ -6006,11 +6034,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -6019,11 +6047,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -6032,11 +6060,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -6045,11 +6073,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-24
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC7AA83-347F-4963-8DFC-BB66E13E1DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA471284-70B1-4AD8-8EE9-F55443AB3F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2203" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2207" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5730,7 +5730,9 @@
       <c r="AB3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC3" s="2"/>
+      <c r="AC3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
@@ -5810,7 +5812,9 @@
       <c r="AB4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC4" s="2"/>
+      <c r="AC4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
@@ -5890,7 +5894,9 @@
       <c r="AB5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC5" s="2"/>
+      <c r="AC5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
@@ -5970,7 +5976,9 @@
       <c r="AB6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC6" s="2"/>
+      <c r="AC6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
@@ -6034,7 +6042,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6047,7 +6055,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6060,7 +6068,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6077,7 +6085,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-26
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA471284-70B1-4AD8-8EE9-F55443AB3F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCF5037-5C9B-4446-B80B-FD876E85A4FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2207" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2219" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5733,9 +5733,15 @@
       <c r="AC3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD3" s="2"/>
-      <c r="AE3" s="2"/>
-      <c r="AF3" s="2"/>
+      <c r="AD3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AG3" s="7"/>
       <c r="AH3" s="7"/>
       <c r="AI3" s="2"/>
@@ -5815,9 +5821,15 @@
       <c r="AC4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD4" s="2"/>
-      <c r="AE4" s="2"/>
-      <c r="AF4" s="2"/>
+      <c r="AD4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
       <c r="AI4" s="2"/>
@@ -5897,9 +5909,15 @@
       <c r="AC5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD5" s="2"/>
-      <c r="AE5" s="2"/>
-      <c r="AF5" s="2"/>
+      <c r="AD5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AG5" s="7"/>
       <c r="AH5" s="7"/>
       <c r="AI5" s="2"/>
@@ -5979,9 +5997,15 @@
       <c r="AC6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AD6" s="2"/>
-      <c r="AE6" s="2"/>
-      <c r="AF6" s="2"/>
+      <c r="AD6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AG6" s="7"/>
       <c r="AH6" s="7"/>
       <c r="AI6" s="2"/>
@@ -6042,11 +6066,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -6055,11 +6079,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -6068,11 +6092,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -6081,11 +6105,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-30
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCF5037-5C9B-4446-B80B-FD876E85A4FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E1A587-DAED-4BF4-A515-3A914B27C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2219" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2223" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5447,6 +5447,7 @@
     <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
@@ -5744,7 +5745,9 @@
       </c>
       <c r="AG3" s="7"/>
       <c r="AH3" s="7"/>
-      <c r="AI3" s="2"/>
+      <c r="AI3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AJ3" s="2"/>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
@@ -5832,7 +5835,9 @@
       </c>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
-      <c r="AI4" s="2"/>
+      <c r="AI4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AJ4" s="2"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
@@ -5920,7 +5925,9 @@
       </c>
       <c r="AG5" s="7"/>
       <c r="AH5" s="7"/>
-      <c r="AI5" s="2"/>
+      <c r="AI5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AJ5" s="2"/>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
@@ -6008,7 +6015,9 @@
       </c>
       <c r="AG6" s="7"/>
       <c r="AH6" s="7"/>
-      <c r="AI6" s="2"/>
+      <c r="AI6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AJ6" s="2"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Daily attendance update - 2026-03-31
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E1A587-DAED-4BF4-A515-3A914B27C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847CF732-1047-4093-B7DA-BC7F0D1F8224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2223" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2227" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -5748,7 +5748,9 @@
       <c r="AI3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AJ3" s="2"/>
+      <c r="AJ3" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -5838,7 +5840,9 @@
       <c r="AI4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AJ4" s="2"/>
+      <c r="AJ4" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -5928,7 +5932,9 @@
       <c r="AI5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AJ5" s="2"/>
+      <c r="AJ5" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -6018,7 +6024,9 @@
       <c r="AI6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AJ6" s="2"/>
+      <c r="AJ6" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-01
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847CF732-1047-4093-B7DA-BC7F0D1F8224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E792496-8C59-4419-8AA5-29D088F3EC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="14" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -28,6 +28,7 @@
     <sheet name="UV-WMS Admin January 2026" sheetId="13" r:id="rId13"/>
     <sheet name="UV-WMS Admin February 2026" sheetId="14" r:id="rId14"/>
     <sheet name="UV-WMS Admin March 2026" sheetId="15" r:id="rId15"/>
+    <sheet name="UV-WMS Admin April 2026" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2227" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2289" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -361,7 +362,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="37">
+  <dxfs count="40">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2579,13 +2610,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3277,13 +3308,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4011,13 +4042,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4737,13 +4768,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5413,13 +5444,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6082,8 +6113,8 @@
         <v>12</v>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(F3:AG3,"WFO")</f>
-        <v>12</v>
+        <f>COUNTIF(F3:AJ3,"WFO")</f>
+        <v>13</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6095,8 +6126,8 @@
         <v>19</v>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(F4:AG4,"WFO")</f>
-        <v>13</v>
+        <f>COUNTIF(F4:AJ4,"WFO")</f>
+        <v>15</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6108,8 +6139,8 @@
         <v>20</v>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(F5:AG5,"WFO")</f>
-        <v>11</v>
+        <f>COUNTIF(F5:AJ5,"WFO")</f>
+        <v>12</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6121,12 +6152,559 @@
         <v>23</v>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(F6:AG6,"WFO")</f>
-        <v>13</v>
+        <f>COUNTIF(F6:AJ6,"WFO")</f>
+        <v>15</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
         <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B12:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
+  <dimension ref="A1:AI15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46113</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46114</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46115</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46116</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46117</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46118</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46119</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46120</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46121</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46122</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46123</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46124</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46125</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46126</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46127</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46128</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46129</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46130</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46131</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46132</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46133</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46134</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46135</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46136</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46137</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46138</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46139</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46140</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46141</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="7"/>
+      <c r="AE3" s="7"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="7"/>
+      <c r="AE4" s="7"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="7"/>
+      <c r="AE5" s="7"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="7"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="7"/>
+      <c r="AE6" s="7"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+    </row>
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF(F3:AI3,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIF(F3:AG3,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F4:AI4,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(F4:AG4,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(F6:AG6,"WFH")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7589,10 +8167,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="36" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="39" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8304,10 +8882,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="34" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9029,15 +9607,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="32" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="30" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9726,13 +10304,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10449,13 +11027,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11159,13 +11737,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11866,13 +12444,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-02
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E792496-8C59-4419-8AA5-29D088F3EC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5109C66-C4A1-4BED-A478-D193793B0D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2289" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2305" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6430,11 +6430,17 @@
       <c r="F3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="G3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -6479,15 +6485,29 @@
       <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="K4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="2"/>
@@ -6528,11 +6548,17 @@
       <c r="F5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="G5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -6577,11 +6603,17 @@
       <c r="F6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="G6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -6661,11 +6693,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -6674,11 +6706,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -6687,11 +6719,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -6700,7 +6732,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-07
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5109C66-C4A1-4BED-A478-D193793B0D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B520326-F967-4EE8-AFDA-5656E8C97EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2305" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2308" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -1094,31 +1094,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1328,7 +1328,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1422,7 +1422,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1861,7 +1861,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1890,30 +1890,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2123,7 +2123,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2405,7 +2405,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2537,7 +2537,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2627,26 +2627,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2850,7 +2850,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2937,7 +2937,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3024,7 +3024,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3111,7 +3111,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3198,7 +3198,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3235,7 +3235,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3325,27 +3325,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3455,7 +3455,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3555,7 +3555,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3931,7 +3931,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3969,7 +3969,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4059,27 +4059,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4289,7 +4289,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4695,7 +4695,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4706,7 +4706,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4732,7 +4732,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4745,7 +4745,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4785,26 +4785,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4905,7 +4905,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4996,7 +4996,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5371,7 +5371,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5382,7 +5382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5395,7 +5395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5408,7 +5408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5421,7 +5421,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5461,27 +5461,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5691,7 +5691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5875,7 +5875,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5967,7 +5967,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6059,7 +6059,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6097,7 +6097,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6121,7 +6121,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6147,7 +6147,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6187,27 +6187,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6314,7 +6314,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6411,7 +6411,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6441,7 +6441,9 @@
       <c r="K3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L3" s="2"/>
+      <c r="L3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -6466,7 +6468,7 @@
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6529,7 +6531,7 @@
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6559,7 +6561,9 @@
       <c r="K5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="2"/>
+      <c r="L5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -6584,7 +6588,7 @@
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6614,7 +6618,9 @@
       <c r="K6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="2"/>
+      <c r="L6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -6639,7 +6645,7 @@
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6676,7 +6682,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6687,20 +6693,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6713,26 +6719,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -6767,30 +6773,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6891,7 +6897,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6982,7 +6988,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7067,7 +7073,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7154,7 +7160,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7241,7 +7247,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -7326,7 +7332,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -7411,7 +7417,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -7422,7 +7428,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -7435,7 +7441,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -7448,7 +7454,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -7461,7 +7467,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -7474,7 +7480,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -7503,28 +7509,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7634,7 +7640,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7734,7 +7740,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7824,7 +7830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7912,7 +7918,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8000,7 +8006,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8088,7 +8094,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8126,7 +8132,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -8137,7 +8143,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -8150,7 +8156,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -8163,7 +8169,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -8176,7 +8182,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -8214,29 +8220,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8343,7 +8349,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8440,7 +8446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8531,7 +8537,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8622,7 +8628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8713,7 +8719,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8804,7 +8810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8841,7 +8847,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8852,7 +8858,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8865,7 +8871,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8878,7 +8884,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8891,7 +8897,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8929,29 +8935,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9061,7 +9067,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9161,7 +9167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9253,7 +9259,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9345,7 +9351,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9437,7 +9443,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9529,7 +9535,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9566,7 +9572,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9577,7 +9583,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9590,7 +9596,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9603,7 +9609,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9616,7 +9622,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -9658,15 +9664,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9773,7 +9779,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9870,7 +9876,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9959,7 +9965,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10048,7 +10054,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10137,7 +10143,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10226,7 +10232,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10263,7 +10269,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -10274,7 +10280,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10287,7 +10293,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10300,7 +10306,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -10313,7 +10319,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -10353,17 +10359,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10473,7 +10479,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10573,7 +10579,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10667,7 +10673,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10761,7 +10767,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10855,7 +10861,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10949,7 +10955,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10986,7 +10992,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -10997,7 +11003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11010,7 +11016,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11023,7 +11029,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11036,7 +11042,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11076,18 +11082,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11198,7 +11204,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11298,7 +11304,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11388,7 +11394,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11478,7 +11484,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11568,7 +11574,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11658,7 +11664,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11696,7 +11702,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11707,7 +11713,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11720,7 +11726,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11733,7 +11739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11746,7 +11752,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11786,19 +11792,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11905,7 +11911,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12002,7 +12008,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12093,7 +12099,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -12184,7 +12190,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -12275,7 +12281,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -12366,7 +12372,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -12403,7 +12409,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -12414,7 +12420,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -12427,7 +12433,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -12440,7 +12446,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -12453,7 +12459,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-08
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B520326-F967-4EE8-AFDA-5656E8C97EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD813E6C-C2B0-4AA4-816A-A8ADB73D7A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2308" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2311" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6444,7 +6444,9 @@
       <c r="L3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="2"/>
+      <c r="M3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="7"/>
@@ -6564,7 +6566,9 @@
       <c r="L5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="2"/>
+      <c r="M5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="7"/>
@@ -6621,7 +6625,9 @@
       <c r="L6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="2"/>
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="7"/>
@@ -6699,7 +6705,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6729,7 +6735,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.35">
@@ -6738,7 +6744,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-09
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD813E6C-C2B0-4AA4-816A-A8ADB73D7A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B6EC37-244C-4E52-9A17-2884626F4D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2311" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6447,7 +6447,9 @@
       <c r="M3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="2"/>
+      <c r="N3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O3" s="2"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
@@ -6569,7 +6571,9 @@
       <c r="M5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="2"/>
+      <c r="N5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="O5" s="2"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
@@ -6625,10 +6629,12 @@
       <c r="L6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N6" s="2"/>
+      <c r="M6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="O6" s="2"/>
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
@@ -6709,7 +6715,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.35">
@@ -6731,7 +6737,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6748,7 +6754,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-13
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B6EC37-244C-4E52-9A17-2884626F4D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B95105-A306-4C89-B28D-81A6B6661229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2321" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -1094,31 +1094,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1328,7 +1328,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1422,7 +1422,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1516,7 +1516,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1861,7 +1861,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1890,30 +1890,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2123,7 +2123,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2405,7 +2405,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2537,7 +2537,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2627,26 +2627,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2850,7 +2850,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2937,7 +2937,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3024,7 +3024,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3111,7 +3111,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3198,7 +3198,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3235,7 +3235,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3325,27 +3325,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3455,7 +3455,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3555,7 +3555,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3931,7 +3931,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3969,7 +3969,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4059,27 +4059,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4289,7 +4289,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4695,7 +4695,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4706,7 +4706,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4719,7 +4719,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4732,7 +4732,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4745,7 +4745,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4785,26 +4785,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4905,7 +4905,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4996,7 +4996,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5336,7 +5336,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5371,7 +5371,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5382,7 +5382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5395,7 +5395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5408,7 +5408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5421,7 +5421,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5461,27 +5461,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5691,7 +5691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5875,7 +5875,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5967,7 +5967,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6059,7 +6059,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6097,7 +6097,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6121,7 +6121,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6147,7 +6147,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6187,27 +6187,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6314,7 +6314,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6411,7 +6411,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6450,10 +6450,14 @@
       <c r="N3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="2"/>
+      <c r="O3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
-      <c r="R3" s="2"/>
+      <c r="R3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
@@ -6472,7 +6476,7 @@
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6516,7 +6520,9 @@
       </c>
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="2"/>
+      <c r="R4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
@@ -6535,7 +6541,7 @@
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6574,10 +6580,14 @@
       <c r="N5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="2"/>
+      <c r="O5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
-      <c r="R5" s="2"/>
+      <c r="R5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
@@ -6596,7 +6606,7 @@
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6635,10 +6645,14 @@
       <c r="N6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="2"/>
+      <c r="O6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
-      <c r="R6" s="2"/>
+      <c r="R6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -6657,7 +6671,7 @@
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6694,7 +6708,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6705,56 +6719,56 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -6785,30 +6799,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6909,7 +6923,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7000,7 +7014,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7085,7 +7099,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7172,7 +7186,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7259,7 +7273,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -7344,7 +7358,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -7429,7 +7443,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -7440,7 +7454,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -7453,7 +7467,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -7466,7 +7480,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -7479,7 +7493,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -7492,7 +7506,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -7521,28 +7535,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7652,7 +7666,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7752,7 +7766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7842,7 +7856,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7930,7 +7944,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8018,7 +8032,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8106,7 +8120,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8144,7 +8158,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -8155,7 +8169,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -8168,7 +8182,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -8181,7 +8195,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -8194,7 +8208,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -8232,29 +8246,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8361,7 +8375,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8458,7 +8472,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8549,7 +8563,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8640,7 +8654,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8731,7 +8745,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8822,7 +8836,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8859,7 +8873,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8870,7 +8884,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8883,7 +8897,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8896,7 +8910,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8909,7 +8923,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -8947,29 +8961,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9079,7 +9093,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9179,7 +9193,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9271,7 +9285,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9363,7 +9377,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9455,7 +9469,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9547,7 +9561,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9584,7 +9598,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9595,7 +9609,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9608,7 +9622,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9621,7 +9635,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9634,7 +9648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -9676,15 +9690,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9791,7 +9805,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9888,7 +9902,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9977,7 +9991,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10066,7 +10080,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10155,7 +10169,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10244,7 +10258,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10281,7 +10295,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -10292,7 +10306,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -10305,7 +10319,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -10318,7 +10332,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -10331,7 +10345,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -10371,17 +10385,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10491,7 +10505,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10591,7 +10605,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10685,7 +10699,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10779,7 +10793,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10873,7 +10887,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10967,7 +10981,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11004,7 +11018,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11015,7 +11029,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11028,7 +11042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11041,7 +11055,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11054,7 +11068,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11094,18 +11108,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11216,7 +11230,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11316,7 +11330,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11406,7 +11420,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11496,7 +11510,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11586,7 +11600,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11676,7 +11690,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11714,7 +11728,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11725,7 +11739,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11738,7 +11752,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11751,7 +11765,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11764,7 +11778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11804,19 +11818,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11923,7 +11937,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12020,7 +12034,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12111,7 +12125,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -12202,7 +12216,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -12293,7 +12307,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -12384,7 +12398,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -12421,7 +12435,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -12432,7 +12446,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -12445,7 +12459,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -12458,7 +12472,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -12471,7 +12485,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-14
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B95105-A306-4C89-B28D-81A6B6661229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1578EAE8-F506-4574-8D66-9252D7D6A48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2321" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2325" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6458,7 +6458,9 @@
       <c r="R3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S3" s="2"/>
+      <c r="S3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
@@ -6523,7 +6525,9 @@
       <c r="R4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S4" s="2"/>
+      <c r="S4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
@@ -6588,7 +6592,9 @@
       <c r="R5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S5" s="2"/>
+      <c r="S5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
@@ -6653,7 +6659,9 @@
       <c r="R6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S6" s="2"/>
+      <c r="S6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
@@ -6725,7 +6733,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6738,7 +6746,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6751,7 +6759,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6764,7 +6772,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-15
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1578EAE8-F506-4574-8D66-9252D7D6A48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA87D43-FA51-4B8A-AC91-899B914AD77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2325" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2333" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6461,8 +6461,12 @@
       <c r="S3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
+      <c r="T3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V3" s="2"/>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
@@ -6528,8 +6532,12 @@
       <c r="S4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
+      <c r="T4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V4" s="2"/>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
@@ -6595,8 +6603,12 @@
       <c r="S5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
+      <c r="T5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="V5" s="2"/>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
@@ -6662,8 +6674,12 @@
       <c r="S6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
+      <c r="T6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V6" s="2"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
@@ -6733,11 +6749,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -6746,11 +6762,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -6759,11 +6775,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -6772,11 +6788,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-17
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA87D43-FA51-4B8A-AC91-899B914AD77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0577024E-D34B-4508-B0C3-B4EE22BA5CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2333" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2337" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6467,7 +6467,9 @@
       <c r="U3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="V3" s="2"/>
+      <c r="V3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
       <c r="Y3" s="2"/>
@@ -6538,7 +6540,9 @@
       <c r="U4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="V4" s="2"/>
+      <c r="V4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
       <c r="Y4" s="2"/>
@@ -6609,7 +6613,9 @@
       <c r="U5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="V5" s="2"/>
+      <c r="V5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
       <c r="Y5" s="2"/>
@@ -6680,7 +6686,9 @@
       <c r="U6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="V6" s="2"/>
+      <c r="V6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
       <c r="Y6" s="2"/>
@@ -6753,7 +6761,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -6762,7 +6770,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6779,7 +6787,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -6792,7 +6800,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-21
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD850B3-C166-4885-8085-9A2F5E3FE95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A2F268-B40B-4032-9024-C62E63B32A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2337" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2348" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6472,8 +6472,12 @@
       </c>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
+      <c r="Y3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
@@ -6545,8 +6549,12 @@
       </c>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
+      <c r="Y4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
@@ -6618,8 +6626,12 @@
       </c>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
+      <c r="Y5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
       <c r="AC5" s="2"/>
@@ -6691,15 +6703,25 @@
       </c>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
-      <c r="Y6" s="2"/>
-      <c r="Z6" s="2"/>
+      <c r="Y6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
-      <c r="AC6" s="2"/>
+      <c r="AC6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
-      <c r="AF6" s="2"/>
-      <c r="AG6" s="2"/>
+      <c r="AF6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AG6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
     </row>
@@ -6757,7 +6779,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6770,7 +6792,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6783,7 +6805,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6796,7 +6818,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-22
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A2F268-B40B-4032-9024-C62E63B32A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9E1623-5EC4-4CEA-ABC8-16E253F15F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2348" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2352" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6478,7 +6478,9 @@
       <c r="Z3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA3" s="2"/>
+      <c r="AA3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
       <c r="AD3" s="7"/>
@@ -6555,7 +6557,9 @@
       <c r="Z4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="2"/>
+      <c r="AA4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
       <c r="AD4" s="7"/>
@@ -6632,7 +6636,9 @@
       <c r="Z5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA5" s="2"/>
+      <c r="AA5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AB5" s="2"/>
       <c r="AC5" s="2"/>
       <c r="AD5" s="7"/>
@@ -6709,7 +6715,9 @@
       <c r="Z6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA6" s="2"/>
+      <c r="AA6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB6" s="2"/>
       <c r="AC6" s="6" t="s">
         <v>24</v>
@@ -6779,7 +6787,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6792,7 +6800,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6809,7 +6817,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -6818,7 +6826,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-23
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9E1623-5EC4-4CEA-ABC8-16E253F15F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37DB8CC4-ACF7-4ED5-89F6-261875ED016E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2352" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6481,7 +6481,9 @@
       <c r="AA3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB3" s="2"/>
+      <c r="AB3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC3" s="2"/>
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
@@ -6560,7 +6562,9 @@
       <c r="AA4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB4" s="2"/>
+      <c r="AB4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC4" s="2"/>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
@@ -6639,7 +6643,9 @@
       <c r="AA5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AB5" s="2"/>
+      <c r="AB5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC5" s="2"/>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
@@ -6718,7 +6724,9 @@
       <c r="AA6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB6" s="2"/>
+      <c r="AB6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC6" s="6" t="s">
         <v>24</v>
       </c>
@@ -6791,7 +6799,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -6804,7 +6812,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -6813,7 +6821,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -6830,7 +6838,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-27
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37DB8CC4-ACF7-4ED5-89F6-261875ED016E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB63D8A-5B15-491D-BC19-EE2152A9B1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2362" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6484,10 +6484,14 @@
       <c r="AB3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AC3" s="2"/>
+      <c r="AC3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
-      <c r="AF3" s="2"/>
+      <c r="AF3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
@@ -6565,10 +6569,14 @@
       <c r="AB4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AC4" s="2"/>
+      <c r="AC4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
-      <c r="AF4" s="2"/>
+      <c r="AF4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
@@ -6646,10 +6654,14 @@
       <c r="AB5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC5" s="2"/>
+      <c r="AC5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
-      <c r="AF5" s="2"/>
+      <c r="AF5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
@@ -6795,11 +6807,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -6808,11 +6820,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -6821,11 +6833,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-28
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB63D8A-5B15-491D-BC19-EE2152A9B1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8F9882-6A02-4014-A87D-6980764E1DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2362" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2365" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6492,7 +6492,9 @@
       <c r="AF3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG3" s="2"/>
+      <c r="AG3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
     </row>
@@ -6577,7 +6579,9 @@
       <c r="AF4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG4" s="2"/>
+      <c r="AG4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
     </row>
@@ -6662,7 +6666,9 @@
       <c r="AF5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG5" s="2"/>
+      <c r="AG5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
     </row>
@@ -6807,7 +6813,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6820,7 +6826,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6833,7 +6839,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-04-29
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A8F9882-6A02-4014-A87D-6980764E1DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D4AD79-0B46-4B3B-A9AA-DA04302E06E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2365" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2373" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6495,8 +6495,12 @@
       <c r="AG3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH3" s="2"/>
-      <c r="AI3" s="2"/>
+      <c r="AH3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI3" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -6582,8 +6586,12 @@
       <c r="AG4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH4" s="2"/>
-      <c r="AI4" s="2"/>
+      <c r="AH4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI4" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -6669,8 +6677,12 @@
       <c r="AG5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH5" s="2"/>
-      <c r="AI5" s="2"/>
+      <c r="AH5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI5" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -6756,8 +6768,12 @@
       <c r="AG6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AH6" s="2"/>
-      <c r="AI6" s="2"/>
+      <c r="AH6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI6" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -6813,7 +6829,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -6826,7 +6842,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -6852,7 +6868,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-04
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAB2387-F93F-4111-8A52-A21DB51F96E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862A505B-2535-4548-82FD-A96A34DCA9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="15" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <sheet name="UV-WMS Admin February 2026" sheetId="14" r:id="rId14"/>
     <sheet name="UV-WMS Admin March 2026" sheetId="15" r:id="rId15"/>
     <sheet name="UV-WMS Admin April 2026" sheetId="16" r:id="rId16"/>
+    <sheet name="UV-WMS Admin May 2026" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2373" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -362,7 +363,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="40">
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2610,13 +2641,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3308,13 +3339,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4042,13 +4073,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4768,13 +4799,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5444,13 +5475,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6170,13 +6201,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6873,6 +6904,557 @@
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
         <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B12:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
+  <dimension ref="A1:AJ15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46143</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46144</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46145</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46146</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46147</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46148</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46149</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46150</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46151</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46152</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46153</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46154</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46155</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46156</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46157</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46158</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46159</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46160</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46161</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46162</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46163</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46164</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46165</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46166</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46167</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46168</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46169</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46170</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46171</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46172</v>
+      </c>
+      <c r="AJ1" s="1">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="7"/>
+      <c r="AC3" s="7"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="7"/>
+      <c r="AJ3" s="7"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="7"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="7"/>
+      <c r="AC4" s="7"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="7"/>
+      <c r="AJ4" s="7"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="7"/>
+      <c r="AC5" s="7"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="7"/>
+      <c r="AJ5" s="7"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="7"/>
+      <c r="V6" s="7"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="7"/>
+      <c r="AC6" s="7"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="7"/>
+      <c r="AJ6" s="7"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="7"/>
+      <c r="AJ7" s="7"/>
+    </row>
+    <row r="11" spans="1:36" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF(F3:AI3,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIF(F3:AG3,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F4:AI4,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(F4:AG4,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(F6:AG6,"WFH")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8335,10 +8917,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="39" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="42" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9050,10 +9632,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="37" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9775,15 +10357,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="35" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="33" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10472,13 +11054,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11195,13 +11777,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11905,13 +12487,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12612,13 +13194,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-07
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862A505B-2535-4548-82FD-A96A34DCA9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70EF9EA8-C661-41B5-9AA8-F05C945423B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2440" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2456" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -6936,6 +6936,23 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
@@ -7172,10 +7189,18 @@
       <c r="I3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
+      <c r="J3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="2"/>
@@ -7224,10 +7249,18 @@
       <c r="I4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
+      <c r="J4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
       <c r="P4" s="2"/>
@@ -7276,10 +7309,18 @@
       <c r="I5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
+      <c r="J5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="2"/>
@@ -7328,10 +7369,18 @@
       <c r="I6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
+      <c r="J6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="2"/>
@@ -7411,11 +7460,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -7424,11 +7473,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -7437,11 +7486,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -7450,11 +7499,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-08
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70EF9EA8-C661-41B5-9AA8-F05C945423B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089ABB43-5C09-43B7-A9C4-3F3EF9D049EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -7258,8 +7258,8 @@
       <c r="L4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="5" t="s">
-        <v>17</v>
+      <c r="M4" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -7473,11 +7473,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-11
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089ABB43-5C09-43B7-A9C4-3F3EF9D049EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD341EE0-7FD3-4952-9753-B33DFAE49644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2456" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2464" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7203,7 +7203,9 @@
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
-      <c r="P3" s="2"/>
+      <c r="P3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
@@ -7263,7 +7265,9 @@
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
-      <c r="P4" s="2"/>
+      <c r="P4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
@@ -7323,11 +7327,21 @@
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
+      <c r="P5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="U5" s="7"/>
       <c r="V5" s="7"/>
       <c r="W5" s="2"/>
@@ -7383,7 +7397,9 @@
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
-      <c r="P6" s="2"/>
+      <c r="P6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
@@ -7460,7 +7476,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -7473,7 +7489,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7499,7 +7515,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-12
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD341EE0-7FD3-4952-9753-B33DFAE49644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD75FC1-3A5C-457D-8A1F-18B30096881B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2464" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7206,7 +7206,9 @@
       <c r="P3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="2"/>
+      <c r="Q3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
@@ -7268,7 +7270,9 @@
       <c r="P4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="2"/>
+      <c r="Q4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
@@ -7400,7 +7404,9 @@
       <c r="P6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q6" s="2"/>
+      <c r="Q6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
@@ -7476,7 +7482,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -7489,7 +7495,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7515,7 +7521,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-13
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD75FC1-3A5C-457D-8A1F-18B30096881B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87548BD1-2512-41EE-87D3-F351FFF64915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2470" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7209,7 +7209,9 @@
       <c r="Q3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R3" s="2"/>
+      <c r="R3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="7"/>
@@ -7273,7 +7275,9 @@
       <c r="Q4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R4" s="2"/>
+      <c r="R4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4" s="7"/>
@@ -7407,7 +7411,9 @@
       <c r="Q6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R6" s="2"/>
+      <c r="R6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="7"/>
@@ -7482,7 +7488,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -7495,7 +7501,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7521,7 +7527,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-14
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87548BD1-2512-41EE-87D3-F351FFF64915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1411A2B3-85D4-446F-BEEF-4E28EB3F6357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2470" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2473" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7212,7 +7212,9 @@
       <c r="R3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S3" s="2"/>
+      <c r="S3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T3" s="2"/>
       <c r="U3" s="7"/>
       <c r="V3" s="7"/>
@@ -7278,7 +7280,9 @@
       <c r="R4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S4" s="2"/>
+      <c r="S4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T4" s="2"/>
       <c r="U4" s="7"/>
       <c r="V4" s="7"/>
@@ -7414,7 +7418,9 @@
       <c r="R6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S6" s="2"/>
+      <c r="S6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T6" s="2"/>
       <c r="U6" s="7"/>
       <c r="V6" s="7"/>
@@ -7492,7 +7498,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -7505,7 +7511,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -7531,7 +7537,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-15
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1411A2B3-85D4-446F-BEEF-4E28EB3F6357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D85F686-D30C-4004-AF6C-D7CE40ED7559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2473" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7215,7 +7215,9 @@
       <c r="S3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="T3" s="2"/>
+      <c r="T3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U3" s="7"/>
       <c r="V3" s="7"/>
       <c r="W3" s="2"/>
@@ -7283,7 +7285,9 @@
       <c r="S4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="T4" s="2"/>
+      <c r="T4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U4" s="7"/>
       <c r="V4" s="7"/>
       <c r="W4" s="2"/>
@@ -7421,7 +7425,9 @@
       <c r="S6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="T6" s="2"/>
+      <c r="T6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U6" s="7"/>
       <c r="V6" s="7"/>
       <c r="W6" s="2"/>
@@ -7498,7 +7504,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -7507,7 +7513,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7537,7 +7543,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-18
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D85F686-D30C-4004-AF6C-D7CE40ED7559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827A0884-114E-4391-8750-095631980D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2480" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7220,7 +7220,9 @@
       </c>
       <c r="U3" s="7"/>
       <c r="V3" s="7"/>
-      <c r="W3" s="2"/>
+      <c r="W3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
@@ -7290,7 +7292,9 @@
       </c>
       <c r="U4" s="7"/>
       <c r="V4" s="7"/>
-      <c r="W4" s="2"/>
+      <c r="W4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
@@ -7360,7 +7364,9 @@
       </c>
       <c r="U5" s="7"/>
       <c r="V5" s="7"/>
-      <c r="W5" s="2"/>
+      <c r="W5" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="X5" s="2"/>
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
@@ -7430,7 +7436,9 @@
       </c>
       <c r="U6" s="7"/>
       <c r="V6" s="7"/>
-      <c r="W6" s="2"/>
+      <c r="W6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
@@ -7500,7 +7508,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -7513,7 +7521,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7539,7 +7547,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-19
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827A0884-114E-4391-8750-095631980D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B935DDE-E8EE-474E-BFE4-03FEA3682E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2480" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2484" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7223,7 +7223,9 @@
       <c r="W3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X3" s="2"/>
+      <c r="X3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
@@ -7295,7 +7297,9 @@
       <c r="W4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X4" s="2"/>
+      <c r="X4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
       <c r="AA4" s="2"/>
@@ -7367,7 +7371,9 @@
       <c r="W5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="X5" s="2"/>
+      <c r="X5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
       <c r="AA5" s="2"/>
@@ -7439,7 +7445,9 @@
       <c r="W6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X6" s="2"/>
+      <c r="X6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
@@ -7508,7 +7516,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -7521,7 +7529,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7534,7 +7542,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -7547,7 +7555,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-22
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B935DDE-E8EE-474E-BFE4-03FEA3682E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB7CF34-87F4-4AFE-A9EE-A0BAD4337516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2484" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7226,9 +7226,15 @@
       <c r="X3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
+      <c r="Y3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AB3" s="7"/>
       <c r="AC3" s="7"/>
       <c r="AD3" s="2"/>
@@ -7300,9 +7306,15 @@
       <c r="X4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
-      <c r="AA4" s="2"/>
+      <c r="Y4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AB4" s="7"/>
       <c r="AC4" s="7"/>
       <c r="AD4" s="2"/>
@@ -7374,9 +7386,15 @@
       <c r="X5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
-      <c r="AA5" s="2"/>
+      <c r="Y5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AB5" s="7"/>
       <c r="AC5" s="7"/>
       <c r="AD5" s="2"/>
@@ -7448,9 +7466,15 @@
       <c r="X6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Y6" s="2"/>
-      <c r="Z6" s="2"/>
-      <c r="AA6" s="2"/>
+      <c r="Y6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AB6" s="7"/>
       <c r="AC6" s="7"/>
       <c r="AD6" s="2"/>
@@ -7516,11 +7540,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -7529,11 +7553,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -7542,11 +7566,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -7555,11 +7579,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-25
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB7CF34-87F4-4AFE-A9EE-A0BAD4337516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AA26D7-2170-4B46-9D33-CB90AA275BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2500" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -1125,31 +1125,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1359,7 +1359,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1879,7 +1879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1921,30 +1921,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2154,7 +2154,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2568,7 +2568,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2658,26 +2658,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2881,7 +2881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2968,7 +2968,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3055,7 +3055,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3142,7 +3142,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3229,7 +3229,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3266,7 +3266,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3356,27 +3356,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3586,7 +3586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3962,7 +3962,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4000,7 +4000,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4037,7 +4037,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4050,7 +4050,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4090,27 +4090,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4220,7 +4220,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4320,7 +4320,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4726,7 +4726,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4816,26 +4816,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4936,7 +4936,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5027,7 +5027,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5197,7 +5197,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5402,7 +5402,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5413,7 +5413,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5452,7 +5452,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5492,27 +5492,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5622,7 +5622,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5722,7 +5722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5814,7 +5814,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5906,7 +5906,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6090,7 +6090,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6128,7 +6128,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6139,7 +6139,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6165,7 +6165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6178,7 +6178,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6218,27 +6218,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6442,7 +6442,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6533,7 +6533,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6715,7 +6715,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6806,7 +6806,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6843,7 +6843,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6854,7 +6854,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6867,7 +6867,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6880,7 +6880,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6893,7 +6893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6933,29 +6933,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7165,7 +7165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7237,7 +7237,9 @@
       </c>
       <c r="AB3" s="7"/>
       <c r="AC3" s="7"/>
-      <c r="AD3" s="2"/>
+      <c r="AD3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AE3" s="2"/>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
@@ -7245,7 +7247,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7317,7 +7319,9 @@
       </c>
       <c r="AB4" s="7"/>
       <c r="AC4" s="7"/>
-      <c r="AD4" s="2"/>
+      <c r="AD4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AE4" s="2"/>
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
@@ -7325,7 +7329,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7397,7 +7401,9 @@
       </c>
       <c r="AB5" s="7"/>
       <c r="AC5" s="7"/>
-      <c r="AD5" s="2"/>
+      <c r="AD5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
       <c r="AG5" s="2"/>
@@ -7405,7 +7411,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7477,7 +7483,9 @@
       </c>
       <c r="AB6" s="7"/>
       <c r="AC6" s="7"/>
-      <c r="AD6" s="2"/>
+      <c r="AD6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
       <c r="AG6" s="2"/>
@@ -7485,7 +7493,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7523,7 +7531,7 @@
       <c r="AI7" s="7"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="11" spans="1:36" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -7534,52 +7542,52 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -7614,30 +7622,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7738,7 +7746,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7829,7 +7837,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7914,7 +7922,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8001,7 +8009,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8088,7 +8096,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -8173,7 +8181,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -8258,7 +8266,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8269,7 +8277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8282,7 +8290,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8295,7 +8303,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8308,7 +8316,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -8321,7 +8329,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -8350,28 +8358,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8481,7 +8489,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8581,7 +8589,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8671,7 +8679,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8759,7 +8767,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8847,7 +8855,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8935,7 +8943,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8973,7 +8981,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -8984,7 +8992,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -8997,7 +9005,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -9010,7 +9018,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -9023,7 +9031,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -9061,29 +9069,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9190,7 +9198,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9287,7 +9295,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9378,7 +9386,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9469,7 +9477,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9560,7 +9568,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9651,7 +9659,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9688,7 +9696,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9699,7 +9707,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9712,7 +9720,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9725,7 +9733,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9738,7 +9746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -9776,29 +9784,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9908,7 +9916,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10008,7 +10016,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10100,7 +10108,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10192,7 +10200,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10284,7 +10292,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10376,7 +10384,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10413,7 +10421,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -10424,7 +10432,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -10437,7 +10445,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -10450,7 +10458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -10463,7 +10471,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -10505,15 +10513,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10620,7 +10628,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10717,7 +10725,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10806,7 +10814,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10895,7 +10903,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10984,7 +10992,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11073,7 +11081,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11110,7 +11118,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -11121,7 +11129,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11134,7 +11142,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11147,7 +11155,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11160,7 +11168,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11200,17 +11208,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11320,7 +11328,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11420,7 +11428,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11514,7 +11522,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11608,7 +11616,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11702,7 +11710,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11796,7 +11804,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11833,7 +11841,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11844,7 +11852,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11857,7 +11865,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11870,7 +11878,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11883,7 +11891,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11923,18 +11931,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12045,7 +12053,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12145,7 +12153,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12235,7 +12243,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -12325,7 +12333,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -12415,7 +12423,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -12505,7 +12513,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -12543,7 +12551,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -12554,7 +12562,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -12567,7 +12575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -12580,7 +12588,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -12593,7 +12601,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -12633,19 +12641,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12752,7 +12760,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12849,7 +12857,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12940,7 +12948,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13031,7 +13039,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13122,7 +13130,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -13213,7 +13221,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -13250,7 +13258,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -13261,7 +13269,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -13274,7 +13282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -13287,7 +13295,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -13300,7 +13308,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-26
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AA26D7-2170-4B46-9D33-CB90AA275BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439429C6-E564-4F8F-B524-34DED1A0AAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2500" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -1125,31 +1125,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1359,7 +1359,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1879,7 +1879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1921,30 +1921,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2154,7 +2154,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2568,7 +2568,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2658,26 +2658,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2881,7 +2881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2968,7 +2968,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3055,7 +3055,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3142,7 +3142,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3229,7 +3229,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3266,7 +3266,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3356,27 +3356,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3586,7 +3586,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3774,7 +3774,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3962,7 +3962,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4000,7 +4000,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4037,7 +4037,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4050,7 +4050,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4090,27 +4090,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4220,7 +4220,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4320,7 +4320,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4726,7 +4726,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4816,26 +4816,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4936,7 +4936,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5027,7 +5027,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5197,7 +5197,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5282,7 +5282,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5402,7 +5402,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5413,7 +5413,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5439,7 +5439,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5452,7 +5452,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5492,27 +5492,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5622,7 +5622,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5722,7 +5722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5814,7 +5814,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5906,7 +5906,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6090,7 +6090,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6128,7 +6128,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6139,7 +6139,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6165,7 +6165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6178,7 +6178,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6218,27 +6218,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6442,7 +6442,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6533,7 +6533,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6715,7 +6715,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6806,7 +6806,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6843,7 +6843,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6854,7 +6854,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6867,7 +6867,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6880,7 +6880,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6893,7 +6893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6933,29 +6933,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7165,7 +7165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7240,14 +7240,16 @@
       <c r="AD3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE3" s="2"/>
+      <c r="AE3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7322,14 +7324,16 @@
       <c r="AD4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE4" s="2"/>
+      <c r="AE4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7404,14 +7408,16 @@
       <c r="AD5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE5" s="2"/>
+      <c r="AE5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF5" s="2"/>
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7486,14 +7492,16 @@
       <c r="AD6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE6" s="2"/>
+      <c r="AE6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF6" s="2"/>
       <c r="AG6" s="2"/>
       <c r="AH6" s="2"/>
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7531,7 +7539,7 @@
       <c r="AI7" s="7"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -7542,7 +7550,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -7552,42 +7560,42 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -7622,30 +7630,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7746,7 +7754,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7837,7 +7845,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7922,7 +7930,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8009,7 +8017,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8096,7 +8104,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -8181,7 +8189,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -8266,7 +8274,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -8277,7 +8285,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -8290,7 +8298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -8303,7 +8311,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -8316,7 +8324,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -8329,7 +8337,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -8358,28 +8366,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8489,7 +8497,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8589,7 +8597,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -8679,7 +8687,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -8767,7 +8775,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -8855,7 +8863,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -8943,7 +8951,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -8981,7 +8989,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -8992,7 +9000,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -9005,7 +9013,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -9018,7 +9026,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -9031,7 +9039,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -9069,29 +9077,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9198,7 +9206,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9295,7 +9303,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9386,7 +9394,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9477,7 +9485,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9568,7 +9576,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -9659,7 +9667,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -9696,7 +9704,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9707,7 +9715,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9720,7 +9728,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9733,7 +9741,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9746,7 +9754,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -9784,29 +9792,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9916,7 +9924,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10016,7 +10024,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10108,7 +10116,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10200,7 +10208,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10292,7 +10300,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10384,7 +10392,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10421,7 +10429,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -10432,7 +10440,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -10445,7 +10453,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -10458,7 +10466,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -10471,7 +10479,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -10513,15 +10521,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10628,7 +10636,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10725,7 +10733,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10814,7 +10822,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10903,7 +10911,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10992,7 +11000,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11081,7 +11089,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11118,7 +11126,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -11129,7 +11137,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11142,7 +11150,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11155,7 +11163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11168,7 +11176,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11208,17 +11216,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11328,7 +11336,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11428,7 +11436,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11522,7 +11530,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11616,7 +11624,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11710,7 +11718,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11804,7 +11812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11841,7 +11849,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -11852,7 +11860,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -11865,7 +11873,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -11878,7 +11886,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -11891,7 +11899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -11931,18 +11939,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12053,7 +12061,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12153,7 +12161,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12243,7 +12251,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -12333,7 +12341,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -12423,7 +12431,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -12513,7 +12521,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -12551,7 +12559,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -12562,7 +12570,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -12575,7 +12583,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -12588,7 +12596,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -12601,7 +12609,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -12641,19 +12649,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12760,7 +12768,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12857,7 +12865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12948,7 +12956,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13039,7 +13047,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13130,7 +13138,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -13221,7 +13229,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -13258,7 +13266,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -13269,7 +13277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -13282,7 +13290,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -13295,7 +13303,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -13308,7 +13316,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-27
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439429C6-E564-4F8F-B524-34DED1A0AAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C747D3A-F22F-4169-BAA3-A8D894E1ABE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7243,7 +7243,9 @@
       <c r="AE3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AF3" s="2"/>
+      <c r="AF3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
       <c r="AI3" s="7"/>
@@ -7327,7 +7329,9 @@
       <c r="AE4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF4" s="2"/>
+      <c r="AF4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
       <c r="AI4" s="7"/>
@@ -7411,7 +7415,9 @@
       <c r="AE5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF5" s="2"/>
+      <c r="AF5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG5" s="2"/>
       <c r="AH5" s="2"/>
       <c r="AI5" s="7"/>
@@ -7495,7 +7501,9 @@
       <c r="AE6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF6" s="2"/>
+      <c r="AF6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AG6" s="2"/>
       <c r="AH6" s="2"/>
       <c r="AI6" s="7"/>
@@ -7556,7 +7564,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -7569,7 +7577,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -7582,7 +7590,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -7595,7 +7603,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-05-29
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C747D3A-F22F-4169-BAA3-A8D894E1ABE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548FF021-61D3-489E-83C7-4ACA53343C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2516" uniqueCount="29">
   <si>
     <t>Person</t>
   </si>
@@ -7246,8 +7246,12 @@
       <c r="AF3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG3" s="2"/>
-      <c r="AH3" s="2"/>
+      <c r="AG3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
@@ -7332,8 +7336,12 @@
       <c r="AF4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG4" s="2"/>
-      <c r="AH4" s="2"/>
+      <c r="AG4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AH4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
@@ -7418,8 +7426,12 @@
       <c r="AF5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG5" s="2"/>
-      <c r="AH5" s="2"/>
+      <c r="AG5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
@@ -7504,8 +7516,12 @@
       <c r="AF6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AG6" s="2"/>
-      <c r="AH6" s="2"/>
+      <c r="AG6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
@@ -7568,7 +7584,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
@@ -7594,7 +7610,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -7603,11 +7619,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-01
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548FF021-61D3-489E-83C7-4ACA53343C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF91A5F-E2E6-42B1-A451-0C01E39FB735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -30,6 +30,7 @@
     <sheet name="UV-WMS Admin March 2026" sheetId="15" r:id="rId15"/>
     <sheet name="UV-WMS Admin April 2026" sheetId="16" r:id="rId16"/>
     <sheet name="UV-WMS Admin May 2026" sheetId="17" r:id="rId17"/>
+    <sheet name="UV-WMS Admin June 2026" sheetId="18" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2516" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2583" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -139,6 +140,9 @@
   </si>
   <si>
     <t>HOLIDAY</t>
+  </si>
+  <si>
+    <t>Ashish Mohanty</t>
   </si>
 </sst>
 </file>
@@ -363,7 +367,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="43">
+  <dxfs count="46">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2641,13 +2675,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3339,13 +3373,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4073,13 +4107,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4799,13 +4833,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5475,13 +5509,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6201,13 +6235,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6916,13 +6950,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7624,6 +7658,553 @@
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B12:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934EE78C-1B04-4E2F-8C73-18B0A1ECFFAE}">
+  <dimension ref="A1:AI15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46174</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46175</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46176</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46177</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46178</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46179</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46180</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46181</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46182</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46183</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46184</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46185</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46186</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46187</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46188</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46189</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46190</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46191</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46192</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46193</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46194</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46195</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46196</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46197</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46198</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46199</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46200</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46201</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46202</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="7"/>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="7"/>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+    </row>
+    <row r="11" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF(F3:AI3,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIF(F3:AG3,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F4:AI4,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(F4:AG4,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(F6:AG6,"WFH")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9086,10 +9667,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="42" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="45" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9801,10 +10382,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="40" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10526,15 +11107,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="38" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="36" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11223,13 +11804,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11946,13 +12527,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12656,13 +13237,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13363,13 +13944,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-03
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF91A5F-E2E6-42B1-A451-0C01E39FB735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA55DDF-B0E1-47AE-AC0E-35684EEA5290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2583" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2593" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7690,9 +7690,21 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -7918,8 +7930,12 @@
       <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="G3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="7"/>
@@ -7967,8 +7983,12 @@
       <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="7"/>
@@ -8016,8 +8036,12 @@
       <c r="F5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="G5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="7"/>
@@ -8065,8 +8089,12 @@
       <c r="F6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="G6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="7"/>
@@ -8114,8 +8142,12 @@
       <c r="F7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="G7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="7"/>
@@ -8161,11 +8193,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8174,11 +8206,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8187,7 +8219,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -8200,11 +8232,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-05
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA55DDF-B0E1-47AE-AC0E-35684EEA5290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE68922C-C285-41BD-A80D-279EBBC49E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2593" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2603" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7936,8 +7936,12 @@
       <c r="H3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+      <c r="I3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
       <c r="M3" s="2"/>
@@ -7989,8 +7993,12 @@
       <c r="H4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="I4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
       <c r="M4" s="2"/>
@@ -8042,8 +8050,12 @@
       <c r="H5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
+      <c r="I5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
       <c r="M5" s="2"/>
@@ -8095,8 +8107,12 @@
       <c r="H6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="I6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
       <c r="M6" s="2"/>
@@ -8148,8 +8164,12 @@
       <c r="H7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="I7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
       <c r="M7" s="2"/>
@@ -8193,11 +8213,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8210,7 +8230,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8223,7 +8243,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8232,11 +8252,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-10
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE68922C-C285-41BD-A80D-279EBBC49E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{666446E2-9AD4-48FF-ACB2-24B0C4F2217C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2603" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2618" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7944,9 +7944,15 @@
       </c>
       <c r="K3" s="7"/>
       <c r="L3" s="7"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="M3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
       <c r="R3" s="7"/>
@@ -8001,9 +8007,15 @@
       </c>
       <c r="K4" s="7"/>
       <c r="L4" s="7"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="M4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="7"/>
@@ -8058,9 +8070,15 @@
       </c>
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
+      <c r="M5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="7"/>
@@ -8115,9 +8133,15 @@
       </c>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="7"/>
@@ -8172,9 +8196,15 @@
       </c>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
+      <c r="M7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="7"/>
@@ -8213,7 +8243,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
@@ -8226,7 +8256,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -8239,7 +8269,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -8252,7 +8282,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-12
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{666446E2-9AD4-48FF-ACB2-24B0C4F2217C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E3A161-74F2-46C2-A1CF-8E00E1534E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2618" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2628" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7953,8 +7953,12 @@
       <c r="O3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
+      <c r="P3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="R3" s="7"/>
       <c r="S3" s="7"/>
       <c r="T3" s="2"/>
@@ -8016,8 +8020,12 @@
       <c r="O4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
+      <c r="P4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
       <c r="T4" s="2"/>
@@ -8079,8 +8087,12 @@
       <c r="O5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
+      <c r="P5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
       <c r="T5" s="2"/>
@@ -8142,8 +8154,12 @@
       <c r="O6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
+      <c r="P6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
       <c r="T6" s="2"/>
@@ -8205,8 +8221,12 @@
       <c r="O7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
+      <c r="P7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
       <c r="T7" s="2"/>
@@ -8247,7 +8267,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8260,7 +8280,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8273,7 +8293,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8286,7 +8306,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-15
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E3A161-74F2-46C2-A1CF-8E00E1534E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA85C22-B2C5-4A18-B5E8-36183167C651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2628" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2633" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7961,7 +7961,9 @@
       </c>
       <c r="R3" s="7"/>
       <c r="S3" s="7"/>
-      <c r="T3" s="2"/>
+      <c r="T3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
@@ -8028,7 +8030,9 @@
       </c>
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
-      <c r="T4" s="2"/>
+      <c r="T4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
@@ -8095,7 +8099,9 @@
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
-      <c r="T5" s="2"/>
+      <c r="T5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
@@ -8162,7 +8168,9 @@
       </c>
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
-      <c r="T6" s="2"/>
+      <c r="T6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
@@ -8229,7 +8237,9 @@
       </c>
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
-      <c r="T7" s="2"/>
+      <c r="T7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
@@ -8262,12 +8272,12 @@
         <v>12</v>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF(F3:AI3,"WFO")</f>
+        <f>COUNTIF(F4:AI4,"WFO")</f>
+        <v>6</v>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIF(F4:AG4,"WFH")</f>
         <v>5</v>
-      </c>
-      <c r="C12" s="2">
-        <f>COUNTIF(F3:AG3,"WFH")</f>
-        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8275,12 +8285,12 @@
         <v>19</v>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>5</v>
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>7</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>5</v>
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8288,11 +8298,11 @@
         <v>20</v>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>6</v>
+        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <v>7</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <f>COUNTIF(F6:AG6,"WFH")</f>
         <v>4</v>
       </c>
     </row>
@@ -8301,11 +8311,11 @@
         <v>23</v>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <f>COUNTIF(F7:AI7,"WFO")</f>
         <v>6</v>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIF(F6:AG6,"WFH")</f>
+        <f>COUNTIF(F7:AG7,"WFH")</f>
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-17
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62B05A6-DC83-40D4-A004-F469401BADB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B3339B-353C-4754-9749-34279C45F4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2634" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2643" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7964,8 +7964,12 @@
       <c r="T3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
+      <c r="U3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W3" s="2"/>
       <c r="X3" s="2"/>
       <c r="Y3" s="7"/>
@@ -8033,8 +8037,12 @@
       <c r="T4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
+      <c r="U4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
       <c r="Y4" s="7"/>
@@ -8102,8 +8110,12 @@
       <c r="T5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
+      <c r="U5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
       <c r="Y5" s="7"/>
@@ -8171,8 +8183,12 @@
       <c r="T6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
+      <c r="U6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="7"/>
@@ -8243,7 +8259,9 @@
       <c r="U7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="V7" s="2"/>
+      <c r="V7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
       <c r="Y7" s="7"/>
@@ -8275,7 +8293,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -8288,7 +8306,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -8301,11 +8319,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8318,7 +8336,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-18
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B3339B-353C-4754-9749-34279C45F4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080F14F0-C67F-4A4F-9302-D980B43468EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2643" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2648" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7970,7 +7970,9 @@
       <c r="V3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="W3" s="2"/>
+      <c r="W3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X3" s="2"/>
       <c r="Y3" s="7"/>
       <c r="Z3" s="7"/>
@@ -8043,7 +8045,9 @@
       <c r="V4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="W4" s="2"/>
+      <c r="W4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X4" s="2"/>
       <c r="Y4" s="7"/>
       <c r="Z4" s="7"/>
@@ -8116,7 +8120,9 @@
       <c r="V5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="W5" s="2"/>
+      <c r="W5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X5" s="2"/>
       <c r="Y5" s="7"/>
       <c r="Z5" s="7"/>
@@ -8189,7 +8195,9 @@
       <c r="V6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="W6" s="2"/>
+      <c r="W6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X6" s="2"/>
       <c r="Y6" s="7"/>
       <c r="Z6" s="7"/>
@@ -8262,7 +8270,9 @@
       <c r="V7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="W7" s="2"/>
+      <c r="W7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="X7" s="2"/>
       <c r="Y7" s="7"/>
       <c r="Z7" s="7"/>
@@ -8297,7 +8307,7 @@
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8310,7 +8320,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8323,7 +8333,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8332,7 +8342,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-22
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080F14F0-C67F-4A4F-9302-D980B43468EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB5EA6A-8F1C-4E52-8057-C8004D01755C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2648" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2658" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7973,10 +7973,14 @@
       <c r="W3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="X3" s="2"/>
+      <c r="X3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Y3" s="7"/>
       <c r="Z3" s="7"/>
-      <c r="AA3" s="2"/>
+      <c r="AA3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
@@ -8048,10 +8052,14 @@
       <c r="W4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="X4" s="2"/>
+      <c r="X4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Y4" s="7"/>
       <c r="Z4" s="7"/>
-      <c r="AA4" s="2"/>
+      <c r="AA4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
       <c r="AD4" s="2"/>
@@ -8123,10 +8131,14 @@
       <c r="W5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="X5" s="2"/>
+      <c r="X5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Y5" s="7"/>
       <c r="Z5" s="7"/>
-      <c r="AA5" s="2"/>
+      <c r="AA5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB5" s="2"/>
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
@@ -8198,10 +8210,14 @@
       <c r="W6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="X6" s="2"/>
+      <c r="X6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Y6" s="7"/>
       <c r="Z6" s="7"/>
-      <c r="AA6" s="2"/>
+      <c r="AA6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB6" s="2"/>
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
@@ -8273,10 +8289,14 @@
       <c r="W7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X7" s="2"/>
+      <c r="X7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y7" s="7"/>
       <c r="Z7" s="7"/>
-      <c r="AA7" s="2"/>
+      <c r="AA7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
@@ -8286,7 +8306,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -8303,11 +8323,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8316,11 +8336,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8329,11 +8349,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8342,7 +8362,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-23
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB5EA6A-8F1C-4E52-8057-C8004D01755C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5462FF8B-A8E7-4B3F-B5DB-0B3CB4E75F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2658" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2663" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7981,7 +7981,9 @@
       <c r="AA3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB3" s="2"/>
+      <c r="AB3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
@@ -8060,7 +8062,9 @@
       <c r="AA4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB4" s="2"/>
+      <c r="AB4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC4" s="2"/>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
@@ -8139,7 +8143,9 @@
       <c r="AA5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB5" s="2"/>
+      <c r="AB5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
@@ -8218,7 +8224,9 @@
       <c r="AA6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB6" s="2"/>
+      <c r="AB6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
@@ -8297,7 +8305,9 @@
       <c r="AA7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AB7" s="2"/>
+      <c r="AB7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
@@ -8323,7 +8333,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -8336,7 +8346,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -8349,7 +8359,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -8362,7 +8372,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-24
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5462FF8B-A8E7-4B3F-B5DB-0B3CB4E75F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA2EF15-342E-4ECE-AA3C-C3DE23F9886E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2663" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2668" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7984,7 +7984,9 @@
       <c r="AB3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC3" s="2"/>
+      <c r="AC3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
       <c r="AF3" s="7"/>
@@ -8065,7 +8067,9 @@
       <c r="AB4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC4" s="2"/>
+      <c r="AC4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
       <c r="AF4" s="7"/>
@@ -8146,7 +8150,9 @@
       <c r="AB5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC5" s="2"/>
+      <c r="AC5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
       <c r="AF5" s="7"/>
@@ -8227,7 +8233,9 @@
       <c r="AB6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC6" s="2"/>
+      <c r="AC6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
       <c r="AF6" s="7"/>
@@ -8308,7 +8316,9 @@
       <c r="AB7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC7" s="2"/>
+      <c r="AC7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
       <c r="AF7" s="7"/>
@@ -8333,7 +8343,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -8346,7 +8356,7 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -8359,7 +8369,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -8372,7 +8382,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-06-30
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA2EF15-342E-4ECE-AA3C-C3DE23F9886E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C5B788-F194-493A-B9C9-9B3A240406C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2668" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2688" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -7987,12 +7987,20 @@
       <c r="AC3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD3" s="2"/>
-      <c r="AE3" s="2"/>
+      <c r="AD3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AF3" s="7"/>
       <c r="AG3" s="7"/>
-      <c r="AH3" s="2"/>
-      <c r="AI3" s="2"/>
+      <c r="AH3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI3" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -8070,12 +8078,20 @@
       <c r="AC4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD4" s="2"/>
-      <c r="AE4" s="2"/>
+      <c r="AD4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
-      <c r="AH4" s="2"/>
-      <c r="AI4" s="2"/>
+      <c r="AH4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI4" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -8153,12 +8169,20 @@
       <c r="AC5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD5" s="2"/>
-      <c r="AE5" s="2"/>
+      <c r="AD5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AF5" s="7"/>
       <c r="AG5" s="7"/>
-      <c r="AH5" s="2"/>
-      <c r="AI5" s="2"/>
+      <c r="AH5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI5" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -8236,12 +8260,20 @@
       <c r="AC6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD6" s="2"/>
-      <c r="AE6" s="2"/>
+      <c r="AD6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AF6" s="7"/>
       <c r="AG6" s="7"/>
-      <c r="AH6" s="2"/>
-      <c r="AI6" s="2"/>
+      <c r="AH6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI6" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -8319,12 +8351,20 @@
       <c r="AC7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AD7" s="2"/>
-      <c r="AE7" s="2"/>
+      <c r="AD7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AF7" s="7"/>
       <c r="AG7" s="7"/>
-      <c r="AH7" s="2"/>
-      <c r="AI7" s="2"/>
+      <c r="AH7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI7" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
@@ -8343,11 +8383,11 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
@@ -8356,11 +8396,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -8369,11 +8409,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8382,11 +8422,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-01
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C5B788-F194-493A-B9C9-9B3A240406C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87767953-7331-454F-838E-1047A766AEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="17" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -31,6 +31,7 @@
     <sheet name="UV-WMS Admin April 2026" sheetId="16" r:id="rId16"/>
     <sheet name="UV-WMS Admin May 2026" sheetId="17" r:id="rId17"/>
     <sheet name="UV-WMS Admin June 2026" sheetId="18" r:id="rId18"/>
+    <sheet name="UV-WMS Admin July 2026" sheetId="19" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2688" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2756" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -367,7 +368,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="46">
+  <dxfs count="49">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2675,13 +2706,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3373,13 +3404,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4107,13 +4138,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4833,13 +4864,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5509,13 +5540,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6235,13 +6266,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6950,13 +6981,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7670,13 +7701,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8427,6 +8458,576 @@
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B12:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
+  <dimension ref="A1:AJ15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46204</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46205</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46206</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46207</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46208</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46209</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46210</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46211</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46212</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46213</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46214</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46215</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46216</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46217</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46218</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46219</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46220</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46221</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46222</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46223</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46224</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46225</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46226</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46227</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46228</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46229</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46230</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46231</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46232</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46233</v>
+      </c>
+      <c r="AJ1" s="1">
+        <v>46234</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="7"/>
+      <c r="AE3" s="7"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="7"/>
+      <c r="AE4" s="7"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="2"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="7"/>
+      <c r="AE5" s="7"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+      <c r="AJ5" s="2"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="7"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="7"/>
+      <c r="AE6" s="7"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="7"/>
+      <c r="AE7" s="7"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2"/>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF(F4:AI4,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <f>COUNTIF(F4:AG4,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(F6:AG6,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(F7:AG7,"WFH")</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9889,10 +10490,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="45" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="48" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="47" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10604,10 +11205,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="43" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="46" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11329,15 +11930,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="41" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="43" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="39" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12026,13 +12627,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12749,13 +13350,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13459,13 +14060,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14166,13 +14767,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-06
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87767953-7331-454F-838E-1047A766AEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCBB496-08B5-4C95-B45B-3F6D7044617C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2756" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2771" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -1190,31 +1190,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1424,7 +1424,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1612,7 +1612,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1986,30 +1986,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2219,7 +2219,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2501,7 +2501,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2633,7 +2633,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2670,7 +2670,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2723,26 +2723,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2946,7 +2946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3033,7 +3033,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3120,7 +3120,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3207,7 +3207,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3294,7 +3294,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3331,7 +3331,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3421,27 +3421,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3551,7 +3551,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3651,7 +3651,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3839,7 +3839,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4065,7 +4065,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4076,7 +4076,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4089,7 +4089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4115,7 +4115,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4155,27 +4155,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4385,7 +4385,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4791,7 +4791,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4828,7 +4828,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4881,26 +4881,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5092,7 +5092,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5467,7 +5467,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5478,7 +5478,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5504,7 +5504,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5557,27 +5557,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5687,7 +5687,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5787,7 +5787,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5879,7 +5879,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5971,7 +5971,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6155,7 +6155,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6193,7 +6193,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6217,7 +6217,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6230,7 +6230,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6243,7 +6243,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6283,27 +6283,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6410,7 +6410,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6507,7 +6507,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6598,7 +6598,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6689,7 +6689,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6780,7 +6780,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6871,7 +6871,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6908,7 +6908,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6932,7 +6932,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6945,7 +6945,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6958,7 +6958,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6998,29 +6998,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7130,7 +7130,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7230,7 +7230,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7320,7 +7320,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7410,7 +7410,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7500,7 +7500,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7590,7 +7590,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7628,7 +7628,7 @@
       <c r="AI7" s="7"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -7652,7 +7652,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -7678,7 +7678,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -7718,27 +7718,27 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934EE78C-1B04-4E2F-8C73-18B0A1ECFFAE}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7845,7 +7845,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7942,7 +7942,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -8033,7 +8033,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -8124,7 +8124,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -8215,7 +8215,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -8306,7 +8306,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -8397,7 +8397,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -8408,7 +8408,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -8421,7 +8421,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -8434,7 +8434,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -8447,7 +8447,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -8487,27 +8487,27 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8617,7 +8617,7 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8717,7 +8717,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -8736,11 +8736,17 @@
       <c r="F3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="G3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="2"/>
+      <c r="K3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -8767,7 +8773,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -8786,11 +8792,17 @@
       <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="G4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -8817,7 +8829,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -8836,11 +8848,17 @@
       <c r="F5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="G5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -8867,7 +8885,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -8886,11 +8904,17 @@
       <c r="F6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="G6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="2"/>
+      <c r="K6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -8917,7 +8941,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -8936,11 +8960,17 @@
       <c r="F7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="G7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -8967,7 +8997,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -8978,20 +9008,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -9001,33 +9031,33 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -9058,30 +9088,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9182,7 +9212,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9273,7 +9303,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9358,7 +9388,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9445,7 +9475,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9532,7 +9562,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -9617,7 +9647,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -9702,7 +9732,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9713,7 +9743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9726,7 +9756,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9739,7 +9769,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9752,7 +9782,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -9765,7 +9795,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9794,28 +9824,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9925,7 +9955,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10025,7 +10055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10115,7 +10145,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10203,7 +10233,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10291,7 +10321,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10379,7 +10409,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10417,7 +10447,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -10428,7 +10458,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -10441,7 +10471,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -10454,7 +10484,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -10467,7 +10497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -10505,29 +10535,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10634,7 +10664,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10731,7 +10761,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10822,7 +10852,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10913,7 +10943,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11004,7 +11034,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11095,7 +11125,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11132,7 +11162,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -11143,7 +11173,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -11156,7 +11186,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -11169,7 +11199,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -11182,7 +11212,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -11220,29 +11250,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11352,7 +11382,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11452,7 +11482,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11544,7 +11574,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11636,7 +11666,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11728,7 +11758,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11820,7 +11850,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11857,7 +11887,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -11868,7 +11898,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -11881,7 +11911,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -11894,7 +11924,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -11907,7 +11937,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -11949,15 +11979,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12064,7 +12094,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12161,7 +12191,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12250,7 +12280,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -12339,7 +12369,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -12428,7 +12458,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -12517,7 +12547,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -12554,7 +12584,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -12565,7 +12595,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -12578,7 +12608,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -12591,7 +12621,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -12604,7 +12634,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -12644,17 +12674,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12764,7 +12794,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12864,7 +12894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12958,7 +12988,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13052,7 +13082,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13146,7 +13176,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -13240,7 +13270,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -13277,7 +13307,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -13288,7 +13318,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -13301,7 +13331,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -13314,7 +13344,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -13327,7 +13357,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -13367,18 +13397,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -13489,7 +13519,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13589,7 +13619,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -13679,7 +13709,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13769,7 +13799,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13859,7 +13889,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -13949,7 +13979,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -13987,7 +14017,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -13998,7 +14028,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -14011,7 +14041,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -14024,7 +14054,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -14037,7 +14067,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -14077,19 +14107,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -14196,7 +14226,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -14293,7 +14323,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -14384,7 +14414,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -14475,7 +14505,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14566,7 +14596,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14657,7 +14687,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14694,7 +14724,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -14705,7 +14735,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -14718,7 +14748,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -14731,7 +14761,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -14744,7 +14774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-09
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCBB496-08B5-4C95-B45B-3F6D7044617C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68366736-6C0E-4B1E-9077-6F9DD94353FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2771" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2784" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -8747,8 +8747,12 @@
       <c r="K3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
+      <c r="L3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="7"/>
@@ -8803,8 +8807,12 @@
       <c r="K4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
+      <c r="L4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="7"/>
@@ -8859,13 +8867,23 @@
       <c r="K5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
+      <c r="L5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
-      <c r="R5" s="2"/>
+      <c r="R5" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
@@ -8915,8 +8933,12 @@
       <c r="K6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
+      <c r="L6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="7"/>
@@ -8971,8 +8993,12 @@
       <c r="K7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
+      <c r="L7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="7"/>
@@ -9014,7 +9040,7 @@
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
@@ -9031,7 +9057,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.35">
@@ -9040,7 +9066,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
@@ -9053,7 +9079,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-13
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68366736-6C0E-4B1E-9077-6F9DD94353FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BC3AD6-8377-4645-B4A3-775670682F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2784" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2796" uniqueCount="30">
   <si>
     <t>Person</t>
   </si>
@@ -1190,31 +1190,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1424,7 +1424,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1612,7 +1612,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -1986,30 +1986,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2219,7 +2219,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2501,7 +2501,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2633,7 +2633,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2670,7 +2670,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2723,26 +2723,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2946,7 +2946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3033,7 +3033,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3120,7 +3120,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3207,7 +3207,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3294,7 +3294,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3331,7 +3331,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3421,27 +3421,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3551,7 +3551,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3651,7 +3651,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3839,7 +3839,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3933,7 +3933,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4065,7 +4065,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4076,7 +4076,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4089,7 +4089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4115,7 +4115,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4155,27 +4155,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4385,7 +4385,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4791,7 +4791,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4828,7 +4828,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4841,7 +4841,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4881,26 +4881,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5001,7 +5001,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5092,7 +5092,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="AG6" s="7"/>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5467,7 +5467,7 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -5478,7 +5478,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -5491,7 +5491,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -5504,7 +5504,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -5557,27 +5557,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5687,7 +5687,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5787,7 +5787,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5879,7 +5879,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5971,7 +5971,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6155,7 +6155,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6193,7 +6193,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6217,7 +6217,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6230,7 +6230,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6243,7 +6243,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6283,27 +6283,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6410,7 +6410,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6507,7 +6507,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6598,7 +6598,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6689,7 +6689,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6780,7 +6780,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -6871,7 +6871,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -6908,7 +6908,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -6932,7 +6932,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -6945,7 +6945,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -6958,7 +6958,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -6998,29 +6998,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7130,7 +7130,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7230,7 +7230,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -7320,7 +7320,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7410,7 +7410,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7500,7 +7500,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -7590,7 +7590,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7628,7 +7628,7 @@
       <c r="AI7" s="7"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -7639,7 +7639,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -7652,7 +7652,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -7678,7 +7678,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -7718,27 +7718,27 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934EE78C-1B04-4E2F-8C73-18B0A1ECFFAE}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7845,7 +7845,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7942,7 +7942,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -8033,7 +8033,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -8124,7 +8124,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -8215,7 +8215,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -8306,7 +8306,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -8397,7 +8397,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -8408,7 +8408,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -8421,7 +8421,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -8434,7 +8434,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -8447,7 +8447,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -8487,27 +8487,27 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8617,7 +8617,7 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8717,7 +8717,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -8753,11 +8753,17 @@
       <c r="M3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="N3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
-      <c r="R3" s="2"/>
+      <c r="R3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
@@ -8777,7 +8783,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -8813,11 +8819,17 @@
       <c r="M4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="N4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="2"/>
+      <c r="R4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
@@ -8837,7 +8849,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -8903,7 +8915,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -8939,11 +8951,17 @@
       <c r="M6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
+      <c r="N6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
-      <c r="R6" s="2"/>
+      <c r="R6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -8963,7 +8981,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -8999,11 +9017,17 @@
       <c r="M7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
+      <c r="N7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="2"/>
+      <c r="R7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
@@ -9023,7 +9047,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -9034,20 +9058,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="2">
         <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -9060,7 +9084,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -9070,20 +9094,20 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -9114,30 +9138,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9238,7 +9262,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9329,7 +9353,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9414,7 +9438,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9501,7 +9525,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9588,7 +9612,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -9673,7 +9697,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -9758,7 +9782,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9769,7 +9793,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9782,7 +9806,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9795,7 +9819,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9808,7 +9832,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -9821,7 +9845,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9850,28 +9874,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9981,7 +10005,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10081,7 +10105,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10171,7 +10195,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10259,7 +10283,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -10347,7 +10371,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -10435,7 +10459,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -10473,7 +10497,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -10484,7 +10508,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -10497,7 +10521,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -10510,7 +10534,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -10523,7 +10547,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -10561,29 +10585,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10690,7 +10714,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10787,7 +10811,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -10878,7 +10902,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -10969,7 +10993,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11060,7 +11084,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11151,7 +11175,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11188,7 +11212,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -11199,7 +11223,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -11212,7 +11236,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -11225,7 +11249,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -11238,7 +11262,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -11276,29 +11300,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11408,7 +11432,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11508,7 +11532,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -11600,7 +11624,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -11692,7 +11716,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -11784,7 +11808,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -11876,7 +11900,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -11913,7 +11937,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -11924,7 +11948,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -11937,7 +11961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -11950,7 +11974,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -11963,7 +11987,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -12005,15 +12029,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12120,7 +12144,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12217,7 +12241,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -12306,7 +12330,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -12395,7 +12419,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -12484,7 +12508,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -12573,7 +12597,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -12610,7 +12634,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -12621,7 +12645,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -12634,7 +12658,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -12647,7 +12671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -12660,7 +12684,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -12700,17 +12724,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12820,7 +12844,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12920,7 +12944,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -13014,7 +13038,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13108,7 +13132,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13202,7 +13226,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -13296,7 +13320,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -13333,7 +13357,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -13344,7 +13368,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -13357,7 +13381,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -13370,7 +13394,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -13383,7 +13407,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -13423,18 +13447,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -13545,7 +13569,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13645,7 +13669,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -13735,7 +13759,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13825,7 +13849,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13915,7 +13939,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14005,7 +14029,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14043,7 +14067,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -14054,7 +14078,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -14067,7 +14091,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -14080,7 +14104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -14093,7 +14117,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -14133,19 +14157,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -14252,7 +14276,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -14349,7 +14373,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -14440,7 +14464,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -14531,7 +14555,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14622,7 +14646,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14713,7 +14737,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14750,7 +14774,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -14761,7 +14785,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -14774,7 +14798,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -14787,7 +14811,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -14800,7 +14824,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-14
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BC3AD6-8377-4645-B4A3-775670682F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC30B96A-CA6C-4BD2-A908-8A72AA110882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2796" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2812" uniqueCount="31">
   <si>
     <t>Person</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>Ashish Mohanty</t>
+  </si>
+  <si>
+    <t>Anuj</t>
   </si>
 </sst>
 </file>
@@ -8486,7 +8489,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
-  <dimension ref="A1:AJ15"/>
+  <dimension ref="A1:AJ16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -8518,7 +8521,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E1" s="10" t="s">
         <v>4</v>
@@ -8719,10 +8722,10 @@
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2">
-        <v>35898</v>
+        <v>51690</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -8733,19 +8736,13 @@
       <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="5" t="s">
-        <v>17</v>
+      <c r="K3" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="L3" s="4" t="s">
         <v>16</v>
@@ -8764,7 +8761,9 @@
       <c r="R3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S3" s="2"/>
+      <c r="S3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
@@ -8785,7 +8784,7 @@
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2">
         <v>35898</v>
@@ -8799,8 +8798,8 @@
       <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>16</v>
+      <c r="F4" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>17</v>
@@ -8810,8 +8809,8 @@
       </c>
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="4" t="s">
-        <v>16</v>
+      <c r="K4" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="L4" s="4" t="s">
         <v>16</v>
@@ -8830,7 +8829,9 @@
       <c r="R4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S4" s="2"/>
+      <c r="S4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
@@ -8851,10 +8852,10 @@
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2">
-        <v>33548</v>
+        <v>35898</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>13</v>
@@ -8876,14 +8877,14 @@
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>17</v>
+      <c r="K5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>17</v>
@@ -8893,10 +8894,12 @@
       </c>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
-      <c r="R5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="S5" s="2"/>
+      <c r="R5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
@@ -8917,10 +8920,10 @@
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="2">
-        <v>44429</v>
+        <v>33548</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>13</v>
@@ -8929,7 +8932,7 @@
         <v>14</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>16</v>
@@ -8942,14 +8945,14 @@
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>16</v>
+      <c r="K6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>17</v>
@@ -8962,7 +8965,9 @@
       <c r="R6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="S6" s="2"/>
+      <c r="S6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
@@ -8983,10 +8988,10 @@
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2">
-        <v>45078</v>
+        <v>44429</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>13</v>
@@ -8997,8 +9002,8 @@
       <c r="E7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>17</v>
+      <c r="F7" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>17</v>
@@ -9025,10 +9030,12 @@
       </c>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="S7" s="2"/>
+      <c r="R7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="S7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
@@ -9047,66 +9054,134 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="7"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="7"/>
+      <c r="AE8" s="7"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2"/>
+      <c r="AJ8" s="2"/>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="2">
-        <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>5</v>
-      </c>
-      <c r="C12" s="2">
-        <f>COUNTIF(F4:AG4,"WFH")</f>
-        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="2">
+        <f>COUNTIF(F8:AI8,"WFO")</f>
+        <v>5</v>
+      </c>
+      <c r="C16" s="2">
+        <f>COUNTIF(F8:AG8,"WFH")</f>
         <v>5</v>
       </c>
     </row>
@@ -9119,7 +9194,7 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="B12:B15">
+  <conditionalFormatting sqref="B13:B16">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-17
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC30B96A-CA6C-4BD2-A908-8A72AA110882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D8B08E-3DB3-4327-AB21-3109252F4C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2812" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2830" uniqueCount="31">
   <si>
     <t>Person</t>
   </si>
@@ -8764,9 +8764,15 @@
       <c r="S3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
+      <c r="T3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
       <c r="Y3" s="2"/>
@@ -8832,9 +8838,15 @@
       <c r="S4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
+      <c r="T4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
       <c r="Y4" s="2"/>
@@ -8900,9 +8912,15 @@
       <c r="S5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
+      <c r="T5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
       <c r="Y5" s="2"/>
@@ -8968,9 +8986,15 @@
       <c r="S6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
+      <c r="T6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
       <c r="Y6" s="2"/>
@@ -9036,9 +9060,15 @@
       <c r="S7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
+      <c r="T7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W7" s="7"/>
       <c r="X7" s="7"/>
       <c r="Y7" s="2"/>
@@ -9104,9 +9134,15 @@
       <c r="S8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
+      <c r="T8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
       <c r="Y8" s="2"/>
@@ -9139,11 +9175,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -9152,11 +9188,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -9165,11 +9201,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:36" x14ac:dyDescent="0.25">
@@ -9178,11 +9214,11 @@
       </c>
       <c r="B16" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2">
         <f>COUNTIF(F8:AG8,"WFH")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-23
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D8B08E-3DB3-4327-AB21-3109252F4C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A757A2-7AEA-4669-98AF-BCFFBBF263A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2830" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>Anuj</t>
+  </si>
+  <si>
+    <t>Pradeep S</t>
   </si>
 </sst>
 </file>
@@ -8489,7 +8492,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
-  <dimension ref="A1:AJ16"/>
+  <dimension ref="A1:AJ17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -8775,10 +8778,18 @@
       </c>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
+      <c r="Y3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC3" s="2"/>
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
@@ -8849,10 +8860,18 @@
       </c>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
-      <c r="AA4" s="2"/>
-      <c r="AB4" s="2"/>
+      <c r="Y4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC4" s="2"/>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
@@ -8923,10 +8942,18 @@
       </c>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
-      <c r="AA5" s="2"/>
-      <c r="AB5" s="2"/>
+      <c r="Y5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC5" s="2"/>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
@@ -8938,10 +8965,10 @@
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2">
-        <v>33548</v>
+        <v>51693</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>13</v>
@@ -8952,55 +8979,37 @@
       <c r="E6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
       <c r="I6" s="7"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
-      <c r="R6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="S6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="T6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="U6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="V6" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
-      <c r="Y6" s="2"/>
-      <c r="Z6" s="2"/>
-      <c r="AA6" s="2"/>
-      <c r="AB6" s="2"/>
+      <c r="Y6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC6" s="2"/>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
@@ -9012,10 +9021,10 @@
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" s="2">
-        <v>44429</v>
+        <v>33548</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>13</v>
@@ -9024,7 +9033,7 @@
         <v>14</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>16</v>
@@ -9037,14 +9046,14 @@
       </c>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>16</v>
+      <c r="K7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>17</v>
@@ -9066,15 +9075,23 @@
       <c r="U7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="V7" s="5" t="s">
-        <v>17</v>
+      <c r="V7" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="W7" s="7"/>
       <c r="X7" s="7"/>
-      <c r="Y7" s="2"/>
-      <c r="Z7" s="2"/>
-      <c r="AA7" s="2"/>
-      <c r="AB7" s="2"/>
+      <c r="Y7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC7" s="2"/>
       <c r="AD7" s="7"/>
       <c r="AE7" s="7"/>
@@ -9086,10 +9103,10 @@
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" s="2">
-        <v>45078</v>
+        <v>44429</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>13</v>
@@ -9100,8 +9117,8 @@
       <c r="E8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>17</v>
+      <c r="F8" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>17</v>
@@ -9128,8 +9145,8 @@
       </c>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="4" t="s">
-        <v>16</v>
+      <c r="R8" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="S8" s="4" t="s">
         <v>16</v>
@@ -9145,10 +9162,18 @@
       </c>
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2"/>
-      <c r="AA8" s="2"/>
-      <c r="AB8" s="2"/>
+      <c r="Y8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AC8" s="2"/>
       <c r="AD8" s="7"/>
       <c r="AE8" s="7"/>
@@ -9158,67 +9183,149 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="2"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="2">
+        <v>45078</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
+      <c r="R9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="T9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="U9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W9" s="7"/>
+      <c r="X9" s="7"/>
+      <c r="Y9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AC9" s="2"/>
+      <c r="AD9" s="7"/>
+      <c r="AE9" s="7"/>
+      <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="2"/>
+      <c r="AI9" s="2"/>
+      <c r="AJ9" s="2"/>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2">
-        <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>7</v>
-      </c>
-      <c r="C13" s="2">
-        <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(F6:AI6,"WFO")</f>
-        <v>4</v>
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>10</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIF(F6:AG6,"WFH")</f>
-        <v>8</v>
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B16" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C16" s="2">
         <f>COUNTIF(F8:AG8,"WFH")</f>
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2">
+        <f>COUNTIF(F9:AI9,"WFO")</f>
+        <v>8</v>
+      </c>
+      <c r="C17" s="2">
+        <f>COUNTIF(F9:AG9,"WFH")</f>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -9230,7 +9337,7 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="B13:B16">
+  <conditionalFormatting sqref="B14:B17">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>

</xml_diff>

<commit_message>
Daily attendance update - 2026-07-24
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A757A2-7AEA-4669-98AF-BCFFBBF263A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF47F21-05A3-46B3-8546-69B33D38D2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2869" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -8790,7 +8790,9 @@
       <c r="AB3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AC3" s="2"/>
+      <c r="AC3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
       <c r="AF3" s="2"/>
@@ -8872,7 +8874,9 @@
       <c r="AB4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AC4" s="2"/>
+      <c r="AC4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="2"/>
@@ -8954,7 +8958,9 @@
       <c r="AB5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AC5" s="2"/>
+      <c r="AC5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
       <c r="AF5" s="2"/>
@@ -8968,7 +8974,7 @@
         <v>31</v>
       </c>
       <c r="B6" s="2">
-        <v>51693</v>
+        <v>52370</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>13</v>
@@ -9010,7 +9016,9 @@
       <c r="AB6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC6" s="2"/>
+      <c r="AC6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="2"/>
@@ -9092,7 +9100,9 @@
       <c r="AB7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC7" s="2"/>
+      <c r="AC7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AD7" s="7"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="2"/>
@@ -9174,7 +9184,9 @@
       <c r="AB8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AC8" s="2"/>
+      <c r="AC8" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="AD8" s="7"/>
       <c r="AE8" s="7"/>
       <c r="AF8" s="2"/>
@@ -9256,7 +9268,9 @@
       <c r="AB9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="AC9" s="2"/>
+      <c r="AC9" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="AD9" s="7"/>
       <c r="AE9" s="7"/>
       <c r="AF9" s="2"/>
@@ -9286,7 +9300,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -9295,7 +9309,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-08-03
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF47F21-05A3-46B3-8546-69B33D38D2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC6B802-2AA4-4513-8B7C-7ACCE1EF9FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -32,6 +32,7 @@
     <sheet name="UV-WMS Admin May 2026" sheetId="17" r:id="rId17"/>
     <sheet name="UV-WMS Admin June 2026" sheetId="18" r:id="rId18"/>
     <sheet name="UV-WMS Admin July 2026" sheetId="19" r:id="rId19"/>
+    <sheet name="UV-WMS Admin Aug 2026" sheetId="20" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2869" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2971" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -374,7 +375,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="49">
+  <dxfs count="52">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2712,13 +2743,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3410,13 +3441,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4144,13 +4175,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4870,13 +4901,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5546,13 +5577,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6272,13 +6303,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6987,13 +7018,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7707,13 +7738,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8476,13 +8507,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8795,11 +8826,21 @@
       </c>
       <c r="AD3" s="7"/>
       <c r="AE3" s="7"/>
-      <c r="AF3" s="2"/>
-      <c r="AG3" s="2"/>
-      <c r="AH3" s="2"/>
-      <c r="AI3" s="2"/>
-      <c r="AJ3" s="2"/>
+      <c r="AF3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ3" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -8879,11 +8920,21 @@
       </c>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
-      <c r="AF4" s="2"/>
-      <c r="AG4" s="2"/>
-      <c r="AH4" s="2"/>
-      <c r="AI4" s="2"/>
-      <c r="AJ4" s="2"/>
+      <c r="AF4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ4" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -8963,11 +9014,21 @@
       </c>
       <c r="AD5" s="7"/>
       <c r="AE5" s="7"/>
-      <c r="AF5" s="2"/>
-      <c r="AG5" s="2"/>
-      <c r="AH5" s="2"/>
-      <c r="AI5" s="2"/>
-      <c r="AJ5" s="2"/>
+      <c r="AF5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ5" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -9021,11 +9082,21 @@
       </c>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
-      <c r="AF6" s="2"/>
-      <c r="AG6" s="2"/>
-      <c r="AH6" s="2"/>
-      <c r="AI6" s="2"/>
-      <c r="AJ6" s="2"/>
+      <c r="AF6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ6" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -9105,11 +9176,21 @@
       </c>
       <c r="AD7" s="7"/>
       <c r="AE7" s="7"/>
-      <c r="AF7" s="2"/>
-      <c r="AG7" s="2"/>
-      <c r="AH7" s="2"/>
-      <c r="AI7" s="2"/>
-      <c r="AJ7" s="2"/>
+      <c r="AF7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AJ7" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -9189,11 +9270,21 @@
       </c>
       <c r="AD8" s="7"/>
       <c r="AE8" s="7"/>
-      <c r="AF8" s="2"/>
-      <c r="AG8" s="2"/>
-      <c r="AH8" s="2"/>
-      <c r="AI8" s="2"/>
-      <c r="AJ8" s="2"/>
+      <c r="AF8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AJ8" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -9273,8 +9364,12 @@
       </c>
       <c r="AD9" s="7"/>
       <c r="AE9" s="7"/>
-      <c r="AF9" s="2"/>
-      <c r="AG9" s="2"/>
+      <c r="AF9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG9" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH9" s="2"/>
       <c r="AI9" s="2"/>
       <c r="AJ9" s="2"/>
@@ -9296,7 +9391,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
@@ -9322,11 +9417,11 @@
       </c>
       <c r="B16" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2">
         <f>COUNTIF(F8:AG8,"WFH")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -9335,7 +9430,7 @@
       </c>
       <c r="B17" s="2">
         <f>COUNTIF(F9:AI9,"WFO")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C17" s="2">
         <f>COUNTIF(F9:AG9,"WFH")</f>
@@ -9352,13 +9447,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B14:B17">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10102,6 +10197,589 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F59B1450-F750-4AAF-92F1-86BC63885A84}">
+  <dimension ref="A1:AH15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="34" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46237</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46238</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46239</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46240</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46241</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46242</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46243</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46244</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46245</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46246</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46247</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46248</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46249</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46250</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46251</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46252</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46253</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46254</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46255</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46256</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46257</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46258</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46259</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46260</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46261</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46262</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46263</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46264</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2">
+        <v>51690</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="2"/>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="2"/>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="7"/>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="2"/>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>52370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="7"/>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="2"/>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="2"/>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="7"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="2"/>
+      <c r="AE8" s="2"/>
+      <c r="AF8" s="7"/>
+      <c r="AG8" s="7"/>
+      <c r="AH8" s="2"/>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F5:AH5,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(F5:AG5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F7:AH7,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(F7:AG7,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F8:AH8,"WFO")</f>
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(F8:AG8,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B13:B15">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
@@ -10802,10 +11480,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="48" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="51" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="50" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11517,10 +12195,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="46" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="49" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12242,15 +12920,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="44" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="47" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="46" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="42" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12939,13 +13617,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13662,13 +14340,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14372,13 +15050,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15079,13 +15757,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-08-04
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC6B802-2AA4-4513-8B7C-7ACCE1EF9FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5C6AFC-EFE1-4870-B3D8-B53256646E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="18" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" firstSheet="16" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2971" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2977" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -10437,7 +10437,9 @@
       <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -10485,7 +10487,9 @@
       <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -10533,7 +10537,9 @@
       <c r="F5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -10581,7 +10587,9 @@
       <c r="F6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="2"/>
+      <c r="G6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -10629,7 +10637,9 @@
       <c r="F7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -10677,7 +10687,9 @@
       <c r="F8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="2"/>
+      <c r="G8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -10727,7 +10739,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
@@ -10736,7 +10748,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AH7,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(F7:AG7,"WFH")</f>
@@ -10749,7 +10761,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F8:AH8,"WFO")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(F8:AG8,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-08-05
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5C6AFC-EFE1-4870-B3D8-B53256646E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC7DBD3-6789-4FF4-AC9E-738B69593B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" firstSheet="16" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2977" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2987" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -10199,7 +10199,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F59B1450-F750-4AAF-92F1-86BC63885A84}">
-  <dimension ref="A1:AH15"/>
+  <dimension ref="A1:AJ15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -10207,20 +10207,21 @@
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="34" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="16" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10237,188 +10238,200 @@
         <v>4</v>
       </c>
       <c r="F1" s="1">
+        <v>46235</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46236</v>
+      </c>
+      <c r="H1" s="1">
         <v>46237</v>
       </c>
-      <c r="G1" s="1">
+      <c r="I1" s="1">
         <v>46238</v>
       </c>
-      <c r="H1" s="1">
+      <c r="J1" s="1">
         <v>46239</v>
       </c>
-      <c r="I1" s="1">
+      <c r="K1" s="1">
         <v>46240</v>
       </c>
-      <c r="J1" s="1">
+      <c r="L1" s="1">
         <v>46241</v>
       </c>
-      <c r="K1" s="1">
+      <c r="M1" s="1">
         <v>46242</v>
       </c>
-      <c r="L1" s="1">
+      <c r="N1" s="1">
         <v>46243</v>
       </c>
-      <c r="M1" s="1">
+      <c r="O1" s="1">
         <v>46244</v>
       </c>
-      <c r="N1" s="1">
+      <c r="P1" s="1">
         <v>46245</v>
       </c>
-      <c r="O1" s="1">
+      <c r="Q1" s="1">
         <v>46246</v>
       </c>
-      <c r="P1" s="1">
+      <c r="R1" s="1">
         <v>46247</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="S1" s="1">
         <v>46248</v>
       </c>
-      <c r="R1" s="1">
+      <c r="T1" s="1">
         <v>46249</v>
       </c>
-      <c r="S1" s="1">
+      <c r="U1" s="1">
         <v>46250</v>
       </c>
-      <c r="T1" s="1">
+      <c r="V1" s="1">
         <v>46251</v>
       </c>
-      <c r="U1" s="1">
+      <c r="W1" s="1">
         <v>46252</v>
       </c>
-      <c r="V1" s="1">
+      <c r="X1" s="1">
         <v>46253</v>
       </c>
-      <c r="W1" s="1">
+      <c r="Y1" s="1">
         <v>46254</v>
       </c>
-      <c r="X1" s="1">
+      <c r="Z1" s="1">
         <v>46255</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="AA1" s="1">
         <v>46256</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="AB1" s="1">
         <v>46257</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AC1" s="1">
         <v>46258</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AD1" s="1">
         <v>46259</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="AE1" s="1">
         <v>46260</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="AF1" s="1">
         <v>46261</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="AG1" s="1">
         <v>46262</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="AH1" s="1">
         <v>46263</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="AI1" s="1">
         <v>46264</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="AJ1" s="1">
         <v>46265</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="R2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="S2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="R2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="U2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AG2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="AF2" s="1" t="s">
+      <c r="AH2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AG2" s="1" t="s">
+      <c r="AI2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AH2" s="1" t="s">
+      <c r="AJ2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -10434,41 +10447,45 @@
       <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
       <c r="V3" s="2"/>
       <c r="W3" s="2"/>
       <c r="X3" s="2"/>
-      <c r="Y3" s="7"/>
-      <c r="Z3" s="7"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="7"/>
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
-      <c r="AF3" s="7"/>
-      <c r="AG3" s="7"/>
-      <c r="AH3" s="2"/>
-    </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="7"/>
+      <c r="AI3" s="7"/>
+      <c r="AJ3" s="2"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -10484,41 +10501,45 @@
       <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
-      <c r="Y4" s="7"/>
-      <c r="Z4" s="7"/>
-      <c r="AA4" s="2"/>
-      <c r="AB4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="7"/>
+      <c r="AB4" s="7"/>
       <c r="AC4" s="2"/>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
-      <c r="AF4" s="7"/>
-      <c r="AG4" s="7"/>
-      <c r="AH4" s="2"/>
-    </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="7"/>
+      <c r="AI4" s="7"/>
+      <c r="AJ4" s="2"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -10534,41 +10555,49 @@
       <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
-      <c r="R5" s="7"/>
-      <c r="S5" s="7"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="7"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
-      <c r="Y5" s="7"/>
-      <c r="Z5" s="7"/>
-      <c r="AA5" s="2"/>
-      <c r="AB5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="7"/>
+      <c r="AB5" s="7"/>
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
-      <c r="AF5" s="7"/>
-      <c r="AG5" s="7"/>
-      <c r="AH5" s="2"/>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="7"/>
+      <c r="AI5" s="7"/>
+      <c r="AJ5" s="2"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10584,41 +10613,45 @@
       <c r="E6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
-      <c r="R6" s="7"/>
-      <c r="S6" s="7"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="7"/>
+      <c r="U6" s="7"/>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
-      <c r="Y6" s="7"/>
-      <c r="Z6" s="7"/>
-      <c r="AA6" s="2"/>
-      <c r="AB6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="7"/>
+      <c r="AB6" s="7"/>
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
-      <c r="AF6" s="7"/>
-      <c r="AG6" s="7"/>
-      <c r="AH6" s="2"/>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="7"/>
+      <c r="AI6" s="7"/>
+      <c r="AJ6" s="2"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10634,41 +10667,45 @@
       <c r="E7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
-      <c r="R7" s="7"/>
-      <c r="S7" s="7"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="7"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
-      <c r="Y7" s="7"/>
-      <c r="Z7" s="7"/>
-      <c r="AA7" s="2"/>
-      <c r="AB7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="7"/>
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
-      <c r="AF7" s="7"/>
-      <c r="AG7" s="7"/>
-      <c r="AH7" s="2"/>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="7"/>
+      <c r="AI7" s="7"/>
+      <c r="AJ7" s="2"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -10684,41 +10721,45 @@
       <c r="E8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
-      <c r="R8" s="7"/>
-      <c r="S8" s="7"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="7"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
-      <c r="Y8" s="7"/>
-      <c r="Z8" s="7"/>
-      <c r="AA8" s="2"/>
-      <c r="AB8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="7"/>
+      <c r="AB8" s="7"/>
       <c r="AC8" s="2"/>
       <c r="AD8" s="2"/>
       <c r="AE8" s="2"/>
-      <c r="AF8" s="7"/>
-      <c r="AG8" s="7"/>
-      <c r="AH8" s="2"/>
-    </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="7"/>
+      <c r="AI8" s="7"/>
+      <c r="AJ8" s="2"/>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -10729,42 +10770,42 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(F5:AH5,"WFO")</f>
+        <f>COUNTIF(H5:AJ5,"WFO")</f>
+        <v>2</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(H5:AI5,"WFH")</f>
         <v>1</v>
       </c>
-      <c r="C13" s="2">
-        <f>COUNTIF(F5:AG5,"WFH")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(F7:AH7,"WFO")</f>
-        <v>2</v>
+        <f>COUNTIF(H7:AJ7,"WFO")</f>
+        <v>3</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIF(F7:AG7,"WFH")</f>
+        <f>COUNTIF(H7:AI7,"WFH")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(F8:AH8,"WFO")</f>
-        <v>2</v>
+        <f>COUNTIF(H8:AJ8,"WFO")</f>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIF(F8:AG8,"WFH")</f>
+        <f>COUNTIF(H8:AI8,"WFH")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance update - 2026-08-07
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC7DBD3-6789-4FF4-AC9E-738B69593B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9894F6C1-C0C4-42FD-9E7D-1979E2927CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2987" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2997" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -10458,8 +10458,12 @@
       <c r="J3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
+      <c r="K3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
       <c r="O3" s="2"/>
@@ -10512,8 +10516,12 @@
       <c r="J4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="K4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
       <c r="O4" s="2"/>
@@ -10624,8 +10632,12 @@
       <c r="J6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+      <c r="K6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
       <c r="O6" s="2"/>
@@ -10678,8 +10690,12 @@
       <c r="J7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
+      <c r="K7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="2"/>
@@ -10732,8 +10748,12 @@
       <c r="J8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+      <c r="K8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="2"/>
@@ -10789,7 +10809,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(H7:AJ7,"WFO")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
@@ -10806,7 +10826,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-01
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9894F6C1-C0C4-42FD-9E7D-1979E2927CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE160B7-756E-444B-8A8E-CEE8FC3D10E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -33,6 +33,7 @@
     <sheet name="UV-WMS Admin June 2026" sheetId="18" r:id="rId18"/>
     <sheet name="UV-WMS Admin July 2026" sheetId="19" r:id="rId19"/>
     <sheet name="UV-WMS Admin Aug 2026" sheetId="20" r:id="rId20"/>
+    <sheet name="UV-WMS Admin Sep 2026" sheetId="21" r:id="rId21"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -55,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2997" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3164" uniqueCount="32">
   <si>
     <t>Person</t>
   </si>
@@ -226,7 +227,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,6 +264,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -335,7 +342,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -367,6 +374,7 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -375,7 +383,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="52">
+  <dxfs count="55">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2743,13 +2781,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3441,13 +3479,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4175,13 +4213,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4901,13 +4939,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5577,13 +5615,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6303,13 +6341,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7018,13 +7056,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7738,13 +7776,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8507,13 +8545,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9447,13 +9485,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B14:B17">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10212,7 +10250,8 @@
     <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="16" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -10466,28 +10505,60 @@
       </c>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
+      <c r="O3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T3" s="7"/>
       <c r="U3" s="7"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
+      <c r="V3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AA3" s="7"/>
       <c r="AB3" s="7"/>
-      <c r="AC3" s="2"/>
-      <c r="AD3" s="2"/>
-      <c r="AE3" s="2"/>
-      <c r="AF3" s="2"/>
-      <c r="AG3" s="2"/>
+      <c r="AC3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
-      <c r="AJ3" s="2"/>
+      <c r="AJ3" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -10524,28 +10595,60 @@
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
+      <c r="O4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T4" s="7"/>
       <c r="U4" s="7"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
-      <c r="Z4" s="2"/>
+      <c r="V4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="W4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AA4" s="7"/>
       <c r="AB4" s="7"/>
-      <c r="AC4" s="2"/>
-      <c r="AD4" s="2"/>
-      <c r="AE4" s="2"/>
-      <c r="AF4" s="2"/>
-      <c r="AG4" s="2"/>
+      <c r="AC4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
-      <c r="AJ4" s="2"/>
+      <c r="AJ4" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -10582,28 +10685,60 @@
       </c>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
+      <c r="O5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T5" s="7"/>
       <c r="U5" s="7"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
-      <c r="Z5" s="2"/>
+      <c r="V5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="W5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AA5" s="7"/>
       <c r="AB5" s="7"/>
-      <c r="AC5" s="2"/>
-      <c r="AD5" s="2"/>
-      <c r="AE5" s="2"/>
-      <c r="AF5" s="2"/>
-      <c r="AG5" s="2"/>
+      <c r="AC5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
-      <c r="AJ5" s="2"/>
+      <c r="AJ5" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -10640,28 +10775,60 @@
       </c>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
+      <c r="O6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T6" s="7"/>
       <c r="U6" s="7"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
-      <c r="Z6" s="2"/>
+      <c r="V6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="W6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AA6" s="7"/>
       <c r="AB6" s="7"/>
-      <c r="AC6" s="2"/>
-      <c r="AD6" s="2"/>
-      <c r="AE6" s="2"/>
-      <c r="AF6" s="2"/>
-      <c r="AG6" s="2"/>
+      <c r="AC6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
-      <c r="AJ6" s="2"/>
+      <c r="AJ6" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -10698,28 +10865,60 @@
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
+      <c r="O7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T7" s="7"/>
       <c r="U7" s="7"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
-      <c r="Z7" s="2"/>
+      <c r="V7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AA7" s="7"/>
       <c r="AB7" s="7"/>
-      <c r="AC7" s="2"/>
-      <c r="AD7" s="2"/>
-      <c r="AE7" s="2"/>
-      <c r="AF7" s="2"/>
-      <c r="AG7" s="2"/>
+      <c r="AC7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AG7" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="AH7" s="7"/>
       <c r="AI7" s="7"/>
-      <c r="AJ7" s="2"/>
+      <c r="AJ7" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -10756,28 +10955,60 @@
       </c>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
+      <c r="O8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T8" s="7"/>
       <c r="U8" s="7"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
-      <c r="Z8" s="2"/>
+      <c r="V8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="W8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="X8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AA8" s="7"/>
       <c r="AB8" s="7"/>
-      <c r="AC8" s="2"/>
-      <c r="AD8" s="2"/>
-      <c r="AE8" s="2"/>
-      <c r="AF8" s="2"/>
-      <c r="AG8" s="2"/>
+      <c r="AC8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AF8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AH8" s="7"/>
       <c r="AI8" s="7"/>
-      <c r="AJ8" s="2"/>
+      <c r="AJ8" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
@@ -10796,11 +11027,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(H5:AJ5,"WFO")</f>
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -10809,24 +11040,621 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(H7:AJ7,"WFO")</f>
+        <v>10</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(H8:AJ8,"WFO")</f>
+        <v>14</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(H8:AI8,"WFH")</f>
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B13:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57075C38-32AC-4EA3-9612-A4A3D80F7093}">
+  <dimension ref="A1:AI15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46266</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46267</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46268</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46269</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46270</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46271</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46272</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46273</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46274</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46275</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46276</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46277</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46278</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46279</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46280</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46281</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46282</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46283</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46284</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46285</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46286</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46287</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46288</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46289</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46290</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46291</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46292</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46293</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46294</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2">
+        <v>51690</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="15"/>
+      <c r="U3" s="15"/>
+      <c r="V3" s="15"/>
+      <c r="W3" s="15"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="15"/>
+      <c r="AA3" s="15"/>
+      <c r="AB3" s="15"/>
+      <c r="AC3" s="15"/>
+      <c r="AD3" s="15"/>
+      <c r="AE3" s="7"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="15"/>
+      <c r="AH3" s="15"/>
+      <c r="AI3" s="15"/>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="15"/>
+      <c r="U4" s="15"/>
+      <c r="V4" s="15"/>
+      <c r="W4" s="15"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="15"/>
+      <c r="AA4" s="15"/>
+      <c r="AB4" s="15"/>
+      <c r="AC4" s="15"/>
+      <c r="AD4" s="15"/>
+      <c r="AE4" s="7"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="15"/>
+      <c r="AH4" s="15"/>
+      <c r="AI4" s="15"/>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15"/>
+      <c r="V5" s="15"/>
+      <c r="W5" s="15"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="15"/>
+      <c r="AA5" s="15"/>
+      <c r="AB5" s="15"/>
+      <c r="AC5" s="15"/>
+      <c r="AD5" s="15"/>
+      <c r="AE5" s="7"/>
+      <c r="AF5" s="7"/>
+      <c r="AG5" s="15"/>
+      <c r="AH5" s="15"/>
+      <c r="AI5" s="15"/>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>52370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="15"/>
+      <c r="U6" s="15"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="15"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="15"/>
+      <c r="AA6" s="15"/>
+      <c r="AB6" s="15"/>
+      <c r="AC6" s="15"/>
+      <c r="AD6" s="15"/>
+      <c r="AE6" s="7"/>
+      <c r="AF6" s="7"/>
+      <c r="AG6" s="15"/>
+      <c r="AH6" s="15"/>
+      <c r="AI6" s="15"/>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="15"/>
+      <c r="U7" s="15"/>
+      <c r="V7" s="15"/>
+      <c r="W7" s="15"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="15"/>
+      <c r="AA7" s="15"/>
+      <c r="AB7" s="15"/>
+      <c r="AC7" s="15"/>
+      <c r="AD7" s="15"/>
+      <c r="AE7" s="7"/>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="15"/>
+      <c r="AH7" s="15"/>
+      <c r="AI7" s="15"/>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="15"/>
+      <c r="T8" s="15"/>
+      <c r="U8" s="15"/>
+      <c r="V8" s="15"/>
+      <c r="W8" s="15"/>
+      <c r="X8" s="7"/>
+      <c r="Y8" s="7"/>
+      <c r="Z8" s="15"/>
+      <c r="AA8" s="15"/>
+      <c r="AB8" s="15"/>
+      <c r="AC8" s="15"/>
+      <c r="AD8" s="15"/>
+      <c r="AE8" s="7"/>
+      <c r="AF8" s="7"/>
+      <c r="AG8" s="15"/>
+      <c r="AH8" s="15"/>
+      <c r="AI8" s="15"/>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(H5:AI5,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(H7:AI7,"WFO")</f>
+        <v>0</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(H8:AJ8,"WFO")</f>
-        <v>3</v>
+        <f>COUNTIF(H8:AI8,"WFO")</f>
+        <v>0</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -11553,10 +12381,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="51" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="54" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12268,10 +13096,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="49" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="52" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="51" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12993,15 +13821,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="47" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="50" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="49" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="45" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13690,13 +14518,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14413,13 +15241,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15123,13 +15951,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15830,13 +16658,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-02
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101F3365-018E-4EC6-8142-5AB8D7927B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA79DE02-BBBE-45EB-A36A-0A0F6E88C246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3164" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3170" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Pradeep S</t>
+  </si>
+  <si>
+    <t>Holiday</t>
   </si>
 </sst>
 </file>
@@ -359,6 +362,7 @@
     <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -374,7 +378,6 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -1290,19 +1293,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -1400,11 +1403,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -2085,19 +2088,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -2195,11 +2198,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -2818,19 +2821,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -2925,11 +2928,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3517,19 +3520,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -3627,11 +3630,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
@@ -4251,19 +4254,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -4361,11 +4364,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
@@ -4976,19 +4979,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -5077,11 +5080,11 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
@@ -5653,19 +5656,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -5763,11 +5766,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
@@ -6379,19 +6382,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -6486,11 +6489,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -7096,19 +7099,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -7206,11 +7209,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
@@ -7814,19 +7817,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -7921,11 +7924,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
@@ -8583,19 +8586,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -8693,11 +8696,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -9527,19 +9530,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -9628,11 +9631,11 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -10261,19 +10264,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -10371,11 +10374,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -10545,8 +10548,8 @@
       <c r="AD3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE3" s="4" t="s">
-        <v>16</v>
+      <c r="AE3" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="AF3" s="5" t="s">
         <v>17</v>
@@ -10635,8 +10638,8 @@
       <c r="AD4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE4" s="4" t="s">
-        <v>16</v>
+      <c r="AE4" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="AF4" s="5" t="s">
         <v>17</v>
@@ -10697,8 +10700,8 @@
       <c r="R5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S5" s="5" t="s">
-        <v>17</v>
+      <c r="S5" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="T5" s="7"/>
       <c r="U5" s="7"/>
@@ -10725,8 +10728,8 @@
       <c r="AD5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE5" s="4" t="s">
-        <v>16</v>
+      <c r="AE5" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="AF5" s="5" t="s">
         <v>17</v>
@@ -10778,17 +10781,17 @@
       <c r="O6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q6" s="5" t="s">
-        <v>17</v>
+      <c r="P6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S6" s="4" t="s">
-        <v>16</v>
+      <c r="S6" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="T6" s="7"/>
       <c r="U6" s="7"/>
@@ -10815,8 +10818,8 @@
       <c r="AD6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE6" s="4" t="s">
-        <v>16</v>
+      <c r="AE6" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="AF6" s="5" t="s">
         <v>17</v>
@@ -10906,7 +10909,7 @@
         <v>17</v>
       </c>
       <c r="AE7" s="6" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="AF7" s="6" t="s">
         <v>24</v>
@@ -10958,17 +10961,17 @@
       <c r="O8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>17</v>
+      <c r="P8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="R8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="4" t="s">
-        <v>16</v>
+      <c r="S8" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="T8" s="7"/>
       <c r="U8" s="7"/>
@@ -10995,8 +10998,8 @@
       <c r="AD8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AE8" s="4" t="s">
-        <v>16</v>
+      <c r="AE8" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="AF8" s="5" t="s">
         <v>17</v>
@@ -11027,11 +11030,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(H5:AJ5,"WFO")</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
@@ -11053,11 +11056,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(H8:AJ8,"WFO")</f>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -11110,19 +11113,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -11217,11 +11220,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
@@ -11332,35 +11335,37 @@
       <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="S3" s="15"/>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15"/>
-      <c r="V3" s="15"/>
-      <c r="W3" s="15"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
       <c r="X3" s="7"/>
       <c r="Y3" s="7"/>
-      <c r="Z3" s="15"/>
-      <c r="AA3" s="15"/>
-      <c r="AB3" s="15"/>
-      <c r="AC3" s="15"/>
-      <c r="AD3" s="15"/>
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="10"/>
+      <c r="AB3" s="10"/>
+      <c r="AC3" s="10"/>
+      <c r="AD3" s="10"/>
       <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
-      <c r="AG3" s="15"/>
-      <c r="AH3" s="15"/>
-      <c r="AI3" s="15"/>
+      <c r="AG3" s="10"/>
+      <c r="AH3" s="10"/>
+      <c r="AI3" s="10"/>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -11381,35 +11386,37 @@
       <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="G4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
-      <c r="S4" s="15"/>
-      <c r="T4" s="15"/>
-      <c r="U4" s="15"/>
-      <c r="V4" s="15"/>
-      <c r="W4" s="15"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
       <c r="X4" s="7"/>
       <c r="Y4" s="7"/>
-      <c r="Z4" s="15"/>
-      <c r="AA4" s="15"/>
-      <c r="AB4" s="15"/>
-      <c r="AC4" s="15"/>
-      <c r="AD4" s="15"/>
+      <c r="Z4" s="10"/>
+      <c r="AA4" s="10"/>
+      <c r="AB4" s="10"/>
+      <c r="AC4" s="10"/>
+      <c r="AD4" s="10"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
-      <c r="AG4" s="15"/>
-      <c r="AH4" s="15"/>
-      <c r="AI4" s="15"/>
+      <c r="AG4" s="10"/>
+      <c r="AH4" s="10"/>
+      <c r="AI4" s="10"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -11430,35 +11437,37 @@
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="G5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
-      <c r="S5" s="15"/>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
-      <c r="V5" s="15"/>
-      <c r="W5" s="15"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
       <c r="X5" s="7"/>
       <c r="Y5" s="7"/>
-      <c r="Z5" s="15"/>
-      <c r="AA5" s="15"/>
-      <c r="AB5" s="15"/>
-      <c r="AC5" s="15"/>
-      <c r="AD5" s="15"/>
+      <c r="Z5" s="10"/>
+      <c r="AA5" s="10"/>
+      <c r="AB5" s="10"/>
+      <c r="AC5" s="10"/>
+      <c r="AD5" s="10"/>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
-      <c r="AG5" s="15"/>
-      <c r="AH5" s="15"/>
-      <c r="AI5" s="15"/>
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="10"/>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -11479,35 +11488,37 @@
       <c r="F6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="G6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
-      <c r="S6" s="15"/>
-      <c r="T6" s="15"/>
-      <c r="U6" s="15"/>
-      <c r="V6" s="15"/>
-      <c r="W6" s="15"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
       <c r="X6" s="7"/>
       <c r="Y6" s="7"/>
-      <c r="Z6" s="15"/>
-      <c r="AA6" s="15"/>
-      <c r="AB6" s="15"/>
-      <c r="AC6" s="15"/>
-      <c r="AD6" s="15"/>
+      <c r="Z6" s="10"/>
+      <c r="AA6" s="10"/>
+      <c r="AB6" s="10"/>
+      <c r="AC6" s="10"/>
+      <c r="AD6" s="10"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
-      <c r="AG6" s="15"/>
-      <c r="AH6" s="15"/>
-      <c r="AI6" s="15"/>
+      <c r="AG6" s="10"/>
+      <c r="AH6" s="10"/>
+      <c r="AI6" s="10"/>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -11528,35 +11539,37 @@
       <c r="F7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
+      <c r="G7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
-      <c r="N7" s="15"/>
-      <c r="O7" s="15"/>
-      <c r="P7" s="15"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
-      <c r="S7" s="15"/>
-      <c r="T7" s="15"/>
-      <c r="U7" s="15"/>
-      <c r="V7" s="15"/>
-      <c r="W7" s="15"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
+      <c r="W7" s="10"/>
       <c r="X7" s="7"/>
       <c r="Y7" s="7"/>
-      <c r="Z7" s="15"/>
-      <c r="AA7" s="15"/>
-      <c r="AB7" s="15"/>
-      <c r="AC7" s="15"/>
-      <c r="AD7" s="15"/>
+      <c r="Z7" s="10"/>
+      <c r="AA7" s="10"/>
+      <c r="AB7" s="10"/>
+      <c r="AC7" s="10"/>
+      <c r="AD7" s="10"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
-      <c r="AG7" s="15"/>
-      <c r="AH7" s="15"/>
-      <c r="AI7" s="15"/>
+      <c r="AG7" s="10"/>
+      <c r="AH7" s="10"/>
+      <c r="AI7" s="10"/>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -11577,35 +11590,37 @@
       <c r="F8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
+      <c r="G8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
-      <c r="S8" s="15"/>
-      <c r="T8" s="15"/>
-      <c r="U8" s="15"/>
-      <c r="V8" s="15"/>
-      <c r="W8" s="15"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
       <c r="X8" s="7"/>
       <c r="Y8" s="7"/>
-      <c r="Z8" s="15"/>
-      <c r="AA8" s="15"/>
-      <c r="AB8" s="15"/>
-      <c r="AC8" s="15"/>
-      <c r="AD8" s="15"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="10"/>
+      <c r="AB8" s="10"/>
+      <c r="AC8" s="10"/>
+      <c r="AD8" s="10"/>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
-      <c r="AG8" s="15"/>
-      <c r="AH8" s="15"/>
-      <c r="AI8" s="15"/>
+      <c r="AG8" s="10"/>
+      <c r="AH8" s="10"/>
+      <c r="AI8" s="10"/>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
@@ -11707,19 +11722,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -11817,11 +11832,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -12002,7 +12017,7 @@
       </c>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
-      <c r="AJ3" s="12" t="s">
+      <c r="AJ3" s="13" t="s">
         <v>25</v>
       </c>
     </row>
@@ -12092,7 +12107,7 @@
       </c>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
-      <c r="AJ4" s="13"/>
+      <c r="AJ4" s="14"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -12180,7 +12195,7 @@
       </c>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
-      <c r="AJ5" s="13"/>
+      <c r="AJ5" s="14"/>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -12268,7 +12283,7 @@
       </c>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
-      <c r="AJ6" s="13"/>
+      <c r="AJ6" s="14"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -12306,7 +12321,7 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
-      <c r="AJ7" s="14"/>
+      <c r="AJ7" s="15"/>
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -12419,19 +12434,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -12526,11 +12541,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
@@ -13134,19 +13149,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -13244,11 +13259,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
@@ -13849,19 +13864,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -13956,11 +13971,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
@@ -14546,19 +14561,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -14656,11 +14671,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
@@ -15270,19 +15285,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -15381,11 +15396,11 @@
       <c r="AK1" s="1"/>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
@@ -15981,19 +15996,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -16088,11 +16103,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-03
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64BCDDAA-65ED-428F-8D48-F2DA32873809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A99E08F6-2BA4-4671-AA46-CF596646CBA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3170" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3176" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -11338,7 +11338,9 @@
       <c r="G3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="10"/>
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I3" s="10"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -11389,7 +11391,9 @@
       <c r="G4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I4" s="10"/>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
@@ -11440,7 +11444,9 @@
       <c r="G5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I5" s="10"/>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -11491,7 +11497,9 @@
       <c r="G6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="10"/>
+      <c r="H6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I6" s="10"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
@@ -11542,7 +11550,9 @@
       <c r="G7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="H7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I7" s="10"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
@@ -11593,7 +11603,9 @@
       <c r="G8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="I8" s="10"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
@@ -11643,7 +11655,7 @@
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -11656,7 +11668,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -11669,7 +11681,7 @@
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>